<commit_message>
Remove MBT, Ernesto Borges e Pessoa & Pessoa de todas as listas
A pedido do usuario, os tres escritorios foram retirados de todas as
planilhas (CSV e XLSX) e bloqueados para nao voltarem em novas coletas.
Base de parcerias: 359 contatos. Base antiga: 396.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S4PddV1zQwAFFfo7t8qVDw
</commit_message>
<xml_diff>
--- a/prospeccao_juridica/RENDA_EXTRA_CONTATOS.xlsx
+++ b/prospeccao_juridica/RENDA_EXTRA_CONTATOS.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="CONTATOS" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONTATOS" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'CONTATOS'!$A$1:$L$111</definedName>
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L111"/>
+  <dimension ref="A1:L110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -3326,12 +3326,12 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>MBT Advogados Associados</t>
+          <t>OAB/RO - Seccional Rondônia</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Ji-Paraná</t>
+          <t>Porto Velho</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
@@ -3346,28 +3346,28 @@
       </c>
       <c r="F49" s="6" t="inlineStr">
         <is>
-          <t>contato@mbtadvocacia.com.br</t>
+          <t>gerencia@oab-ro.org.br</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>Parceria entre escritorios</t>
+          <t>Convenios, credenciamentos e assistencia judiciaria</t>
         </is>
       </c>
       <c r="H49" s="4" t="inlineStr"/>
       <c r="I49" s="4" t="inlineStr">
         <is>
-          <t>https://mbtadvocacia.com.br/</t>
+          <t>https://www.oab-ro.org.br/</t>
         </is>
       </c>
       <c r="J49" s="4" t="inlineStr">
         <is>
-          <t>Tel 69 3421-3130 | Ji-Parana: Av. Ji-Parana, 688, Urupa, CEP 76900-192 | Porto Velho: Av. Carlos Gomes, 513, s-205, Caiari | Vilhena: Av. Barao do Rio Branco, 4174, s-01, Centro | 08h-18h</t>
+          <t>Tel (69) 3217-2100 / (69) 3217-2101 | Rua Paulo Leal, 1300, N. Sra. das Gracas, Porto Velho/RO | Outros e-mails publicados: presidencia@oab-ro.org.br, procuradoria@oab-ro.org.br, protocolo@oab-ro.org.br, ouvidoria@oab-ro.org.br, imprensa@oab-ro.org.br</t>
         </is>
       </c>
       <c r="K49" s="4" t="inlineStr">
         <is>
-          <t>NA SUA CIDADE, com filiais em Porto Velho e Vilhena. O site tem pagina VAGAS propria. Areas: civil, trabalhista, ambiental, tributario, administrativo e COOPERATIVO. Faz recuperacao judicial, falencias e leiloes.</t>
+          <t>CANAL INSTITUCIONAL: a seccional divulga credenciamentos, convenios de assistencia judiciaria e editais. Vale perguntar pela lista de conveniados e pelo cadastro de dativos.</t>
         </is>
       </c>
       <c r="L49" s="4" t="inlineStr">
@@ -3384,12 +3384,12 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>OAB/RO - Seccional Rondônia</t>
+          <t>Reis &amp; Rocha Advogados Associados</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Porto Velho</t>
+          <t>Cacoal</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
@@ -3404,28 +3404,28 @@
       </c>
       <c r="F50" s="6" t="inlineStr">
         <is>
-          <t>gerencia@oab-ro.org.br</t>
+          <t>contato@reiserocha.com.br</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
         <is>
-          <t>Convenios, credenciamentos e assistencia judiciaria</t>
+          <t>Parceria entre escritorios e correspondencia</t>
         </is>
       </c>
       <c r="H50" s="4" t="inlineStr"/>
       <c r="I50" s="4" t="inlineStr">
         <is>
-          <t>https://www.oab-ro.org.br/</t>
+          <t>https://reiserocha.com.br/</t>
         </is>
       </c>
       <c r="J50" s="4" t="inlineStr">
         <is>
-          <t>Tel (69) 3217-2100 / (69) 3217-2101 | Rua Paulo Leal, 1300, N. Sra. das Gracas, Porto Velho/RO | Outros e-mails publicados: presidencia@oab-ro.org.br, procuradoria@oab-ro.org.br, protocolo@oab-ro.org.br, ouvidoria@oab-ro.org.br, imprensa@oab-ro.org.br</t>
+          <t>Tel (69) 3441-2200 | R. Rui Barbosa, 1200, Centro, Cacoal-RO | OAB/RO 190000012-18</t>
         </is>
       </c>
       <c r="K50" s="4" t="inlineStr">
         <is>
-          <t>CANAL INSTITUCIONAL: a seccional divulga credenciamentos, convenios de assistencia judiciaria e editais. Vale perguntar pela lista de conveniados e pelo cadastro de dativos.</t>
+          <t>Areas batem com as suas: bancario, previdenciario, consumidor, tributario, trabalhista. Comarca vizinha.</t>
         </is>
       </c>
       <c r="L50" s="4" t="inlineStr">
@@ -3442,12 +3442,12 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Reis &amp; Rocha Advogados Associados</t>
+          <t>RodaLog Logística</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Cacoal</t>
+          <t>Ji-Paraná</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
@@ -3462,28 +3462,28 @@
       </c>
       <c r="F51" s="6" t="inlineStr">
         <is>
-          <t>contato@reiserocha.com.br</t>
+          <t>atendimento@rodalog.com</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
-          <t>Parceria entre escritorios e correspondencia</t>
+          <t>Assessoria juridica multi-comarca</t>
         </is>
       </c>
       <c r="H51" s="4" t="inlineStr"/>
       <c r="I51" s="4" t="inlineStr">
         <is>
-          <t>https://reiserocha.com.br/</t>
+          <t>https://rodalog.com/</t>
         </is>
       </c>
       <c r="J51" s="4" t="inlineStr">
         <is>
-          <t>Tel (69) 3441-2200 | R. Rui Barbosa, 1200, Centro, Cacoal-RO | OAB/RO 190000012-18</t>
+          <t>Tel (62) 3299-9974 | Matriz Goiania/GO</t>
         </is>
       </c>
       <c r="K51" s="4" t="inlineStr">
         <is>
-          <t>Areas batem com as suas: bancario, previdenciario, consumidor, tributario, trabalhista. Comarca vizinha.</t>
+          <t>FILIAIS EM 10 COMARCAS DE RO: Vilhena, Pimenta Bueno, Cacoal, Presidente Medici, JI-PARANA, Ouro Preto do Oeste, Jaru, Ariquemes, Porto Velho, Guajara-Mirim. Passivo trabalhista e civel espalhado pelo estado.</t>
         </is>
       </c>
       <c r="L51" s="4" t="inlineStr">
@@ -3500,12 +3500,12 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>RodaLog Logística</t>
+          <t>Rolim Net</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Ji-Paraná</t>
+          <t>Rolim de Moura</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
@@ -3520,28 +3520,28 @@
       </c>
       <c r="F52" s="6" t="inlineStr">
         <is>
-          <t>atendimento@rodalog.com</t>
+          <t>contato@rolimnet.com.br</t>
         </is>
       </c>
       <c r="G52" s="4" t="inlineStr">
         <is>
-          <t>Assessoria juridica multi-comarca</t>
+          <t>Defesa em acoes consumeristas nas comarcas de RO</t>
         </is>
       </c>
       <c r="H52" s="4" t="inlineStr"/>
       <c r="I52" s="4" t="inlineStr">
         <is>
-          <t>https://rodalog.com/</t>
+          <t>https://www.rolimnet.com.br/</t>
         </is>
       </c>
       <c r="J52" s="4" t="inlineStr">
         <is>
-          <t>Tel (62) 3299-9974 | Matriz Goiania/GO</t>
+          <t>Tel e WhatsApp (69) 3198-0000 | Av. Manaus, 5095, Centro, Rolim de Moura-RO | CNPJ 09.337.446/0001-80</t>
         </is>
       </c>
       <c r="K52" s="4" t="inlineStr">
         <is>
-          <t>FILIAIS EM 10 COMARCAS DE RO: Vilhena, Pimenta Bueno, Cacoal, Presidente Medici, JI-PARANA, Ouro Preto do Oeste, Jaru, Ariquemes, Porto Velho, Guajara-Mirim. Passivo trabalhista e civel espalhado pelo estado.</t>
+          <t>Provedor com 18 anos atendendo TODO o estado de RO e o Acre. Telecom e um dos setores mais acionados por consumidores (CNJ). Tem pagina Trabalhe Conosco.</t>
         </is>
       </c>
       <c r="L52" s="4" t="inlineStr">
@@ -3558,12 +3558,12 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Rolim Net</t>
+          <t>RondoCoop - Sistema OCB/RO</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Rolim de Moura</t>
+          <t>Porto Velho</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
@@ -3578,28 +3578,28 @@
       </c>
       <c r="F53" s="6" t="inlineStr">
         <is>
-          <t>contato@rolimnet.com.br</t>
+          <t>sistemaocb-ro@rondonia.coop.br</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
-          <t>Defesa em acoes consumeristas nas comarcas de RO</t>
+          <t>Convenio de assessoria juridica cooperativa</t>
         </is>
       </c>
       <c r="H53" s="4" t="inlineStr"/>
       <c r="I53" s="4" t="inlineStr">
         <is>
-          <t>https://www.rolimnet.com.br/</t>
+          <t>https://rondonia.coop.br/rondocoop/</t>
         </is>
       </c>
       <c r="J53" s="4" t="inlineStr">
         <is>
-          <t>Tel e WhatsApp (69) 3198-0000 | Av. Manaus, 5095, Centro, Rolim de Moura-RO | CNPJ 09.337.446/0001-80</t>
+          <t>Tel (69) 99961-4247 / (69) 3224-6116 | R. Paulo Macalao, 4675, Porto Velho</t>
         </is>
       </c>
       <c r="K53" s="4" t="inlineStr">
         <is>
-          <t>Provedor com 18 anos atendendo TODO o estado de RO e o Acre. Telecom e um dos setores mais acionados por consumidores (CNJ). Tem pagina Trabalhe Conosco.</t>
+          <t>Reune +20 cooperativas de RO. Tem pagina de Processos Seletivos e Licitacoes e Contratos.</t>
         </is>
       </c>
       <c r="L53" s="4" t="inlineStr">
@@ -3616,12 +3616,12 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>RondoCoop - Sistema OCB/RO</t>
+          <t>UNICAFES Rondônia</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Porto Velho</t>
+          <t>Ji-Paraná</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
@@ -3636,28 +3636,28 @@
       </c>
       <c r="F54" s="6" t="inlineStr">
         <is>
-          <t>sistemaocb-ro@rondonia.coop.br</t>
+          <t>unicafes@unicafesro.org.br</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr">
         <is>
-          <t>Convenio de assessoria juridica cooperativa</t>
+          <t>Assessoria previdenciaria rural e cooperativa</t>
         </is>
       </c>
       <c r="H54" s="4" t="inlineStr"/>
       <c r="I54" s="4" t="inlineStr">
         <is>
-          <t>https://rondonia.coop.br/rondocoop/</t>
+          <t>https://unicafesro.org.br/quem-somos/</t>
         </is>
       </c>
       <c r="J54" s="4" t="inlineStr">
         <is>
-          <t>Tel (69) 99961-4247 / (69) 3224-6116 | R. Paulo Macalao, 4675, Porto Velho</t>
+          <t>Tel (69) 98462-7685 | Rua Missionaria Gunnar Vingren, 1448, Nova Brasilia, JI-PARANA/RO</t>
         </is>
       </c>
       <c r="K54" s="4" t="inlineStr">
         <is>
-          <t>Reune +20 cooperativas de RO. Tem pagina de Processos Seletivos e Licitacoes e Contratos.</t>
+          <t>SEDE NA SUA CIDADE. Uniao de cooperativas da agricultura familiar - publico direto de previdenciario rural.</t>
         </is>
       </c>
       <c r="L54" s="4" t="inlineStr">
@@ -3674,7 +3674,7 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>UNICAFES Rondônia</t>
+          <t>Mind Consultoria de Gente e Gestão</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
@@ -3687,40 +3687,44 @@
           <t>RO</t>
         </is>
       </c>
-      <c r="E55" s="5" t="inlineStr">
-        <is>
-          <t>E-MAIL</t>
+      <c r="E55" s="9" t="inlineStr">
+        <is>
+          <t>WHATSAPP</t>
         </is>
       </c>
       <c r="F55" s="6" t="inlineStr">
         <is>
-          <t>unicafes@unicafesro.org.br</t>
+          <t>(69) 99220-5249 / (69) 99962-7827</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr">
         <is>
-          <t>Assessoria previdenciaria rural e cooperativa</t>
-        </is>
-      </c>
-      <c r="H55" s="4" t="inlineStr"/>
+          <t>Advogado(a) Associado(a) - Trabalhista Patronal | Ambiental | Civil (PJ)</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
       <c r="I55" s="4" t="inlineStr">
         <is>
-          <t>https://unicafesro.org.br/quem-somos/</t>
+          <t>https://to.indeed.com/aadzhybh6yrx</t>
         </is>
       </c>
       <c r="J55" s="4" t="inlineStr">
         <is>
-          <t>Tel (69) 98462-7685 | Rua Missionaria Gunnar Vingren, 1448, Nova Brasilia, JI-PARANA/RO</t>
+          <t>"Apos realizar sua candidatura pelo site da Solides, envie uma mensagem no WhatsApp: (69) 99220-5249 / (69) 99962-7827. Informar: seu nome + vaga para a qual se candidatou"</t>
         </is>
       </c>
       <c r="K55" s="4" t="inlineStr">
         <is>
-          <t>SEDE NA SUA CIDADE. Uniao de cooperativas da agricultura familiar - publico direto de previdenciario rural.</t>
+          <t>NA SUA CIDADE. Contrato de associacao PJ, R$ 2.500 + bonificacoes. O anuncio diz que NAO buscam perfil de previdenciario - enfatize trabalhista patronal, ambiental e civel.</t>
         </is>
       </c>
       <c r="L55" s="4" t="inlineStr">
         <is>
-          <t>Site institucional (extracao Tavily)</t>
+          <t>Descricao completa da vaga no Indeed (get_job_details)</t>
         </is>
       </c>
     </row>
@@ -3732,12 +3736,12 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>Mind Consultoria de Gente e Gestão</t>
+          <t>Roque &amp; Lima Advocacia</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Ji-Paraná</t>
+          <t>Cacoal</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
@@ -3752,37 +3756,33 @@
       </c>
       <c r="F56" s="6" t="inlineStr">
         <is>
-          <t>(69) 99220-5249 / (69) 99962-7827</t>
+          <t>(69) 98154-8887 / (69) 98428-1401</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
-          <t>Advogado(a) Associado(a) - Trabalhista Patronal | Ambiental | Civil (PJ)</t>
-        </is>
-      </c>
-      <c r="H56" s="4" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>Parceria entre escritorios</t>
+        </is>
+      </c>
+      <c r="H56" s="4" t="inlineStr"/>
       <c r="I56" s="4" t="inlineStr">
         <is>
-          <t>https://to.indeed.com/aadzhybh6yrx</t>
+          <t>https://roqueelimaadvocacia.com.br/sobre/</t>
         </is>
       </c>
       <c r="J56" s="4" t="inlineStr">
         <is>
-          <t>"Apos realizar sua candidatura pelo site da Solides, envie uma mensagem no WhatsApp: (69) 99220-5249 / (69) 99962-7827. Informar: seu nome + vaga para a qual se candidatou"</t>
+          <t>Rua Rio Branco, 2462, Centro, Cacoal/RO | Socios: Dr. Altemir Roque (OAB 1.311), Dra. Cristiane Rodrigues Lima (OAB/RO 7.220), Larissa H Roque (OAB/RO 13.210)</t>
         </is>
       </c>
       <c r="K56" s="4" t="inlineStr">
         <is>
-          <t>NA SUA CIDADE. Contrato de associacao PJ, R$ 2.500 + bonificacoes. O anuncio diz que NAO buscam perfil de previdenciario - enfatize trabalhista patronal, ambiental e civel.</t>
+          <t>ATENCAO: o e-mail do site e hi@example.com - placeholder de template, NAO usar. Contato real e o WhatsApp. Especialistas em Direito Medico e da Saude e Previdenciario - suas areas.</t>
         </is>
       </c>
       <c r="L56" s="4" t="inlineStr">
         <is>
-          <t>Descricao completa da vaga no Indeed (get_job_details)</t>
+          <t>Site institucional (extracao Tavily)</t>
         </is>
       </c>
     </row>
@@ -3794,12 +3794,12 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Roque &amp; Lima Advocacia</t>
+          <t>Covezi Iveco</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>Cacoal</t>
+          <t>Porto Velho</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
@@ -3807,35 +3807,35 @@
           <t>RO</t>
         </is>
       </c>
-      <c r="E57" s="9" t="inlineStr">
-        <is>
-          <t>WHATSAPP</t>
+      <c r="E57" s="7" t="inlineStr">
+        <is>
+          <t>TELEFONE</t>
         </is>
       </c>
       <c r="F57" s="6" t="inlineStr">
         <is>
-          <t>(69) 98154-8887 / (69) 98428-1401</t>
+          <t>(69) 3198-1099</t>
         </is>
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
-          <t>Parceria entre escritorios</t>
+          <t>Assessoria em consumidor, contratos e cobranca</t>
         </is>
       </c>
       <c r="H57" s="4" t="inlineStr"/>
       <c r="I57" s="4" t="inlineStr">
         <is>
-          <t>https://roqueelimaadvocacia.com.br/sobre/</t>
+          <t>https://www.covezi.com.br/</t>
         </is>
       </c>
       <c r="J57" s="4" t="inlineStr">
         <is>
-          <t>Rua Rio Branco, 2462, Centro, Cacoal/RO | Socios: Dr. Altemir Roque (OAB 1.311), Dra. Cristiane Rodrigues Lima (OAB/RO 7.220), Larissa H Roque (OAB/RO 13.210)</t>
+          <t>Central 0800 942 1300 | Filiais RO: PORTO VELHO e VILHENA, ambas (69) 3198-1099 | Matriz Ap. de Goiania/GO | Outras filiais: Anapolis, Itumbiara, Rio Verde, Mineiros, Luziania, Brasilia, Gurupi, Palmas, Araguaina, Marituba/PA</t>
         </is>
       </c>
       <c r="K57" s="4" t="inlineStr">
         <is>
-          <t>ATENCAO: o e-mail do site e hi@example.com - placeholder de template, NAO usar. Contato real e o WhatsApp. Especialistas em Direito Medico e da Saude e Previdenciario - suas areas.</t>
+          <t>DUAS filiais em Rondonia. Tem pagina TRABALHE CONOSCO e FALE CONOSCO. Venda de caminhoes pesados gera contencioso de consumidor, vicio de produto e cobranca.</t>
         </is>
       </c>
       <c r="L57" s="4" t="inlineStr">
@@ -3852,7 +3852,7 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>Covezi Iveco</t>
+          <t>Galvão &amp; Silva Advocacia</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
@@ -3872,28 +3872,28 @@
       </c>
       <c r="F58" s="6" t="inlineStr">
         <is>
-          <t>(69) 3198-1099</t>
+          <t>0800 212 1700</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
-          <t>Assessoria em consumidor, contratos e cobranca</t>
+          <t>Correspondencia nas comarcas do interior de RO</t>
         </is>
       </c>
       <c r="H58" s="4" t="inlineStr"/>
       <c r="I58" s="4" t="inlineStr">
         <is>
-          <t>https://www.covezi.com.br/</t>
+          <t>https://www.galvaoesilva.com/escritorio-de-advocacia-em-porto-velho-ro/</t>
         </is>
       </c>
       <c r="J58" s="4" t="inlineStr">
         <is>
-          <t>Central 0800 942 1300 | Filiais RO: PORTO VELHO e VILHENA, ambas (69) 3198-1099 | Matriz Ap. de Goiania/GO | Outras filiais: Anapolis, Itumbiara, Rio Verde, Mineiros, Luziania, Brasilia, Gurupi, Palmas, Araguaina, Marituba/PA</t>
+          <t>CNPJ 22.889.244/0001-00 | OAB/DF 2609/15</t>
         </is>
       </c>
       <c r="K58" s="4" t="inlineStr">
         <is>
-          <t>DUAS filiais em Rondonia. Tem pagina TRABALHE CONOSCO e FALE CONOSCO. Venda de caminhoes pesados gera contencioso de consumidor, vicio de produto e cobranca.</t>
+          <t>Banca nacional com unidade em Porto Velho. Tem pagina BANCO DE TALENTOS - caminho de entrada.</t>
         </is>
       </c>
       <c r="L58" s="4" t="inlineStr">
@@ -3910,7 +3910,7 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>Galvão &amp; Silva Advocacia</t>
+          <t>Rede Hospitalar Samar</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
@@ -3930,28 +3930,28 @@
       </c>
       <c r="F59" s="6" t="inlineStr">
         <is>
-          <t>0800 212 1700</t>
+          <t>0800 033 0393</t>
         </is>
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
-          <t>Correspondencia nas comarcas do interior de RO</t>
+          <t>Contencioso de saude e trabalhista</t>
         </is>
       </c>
       <c r="H59" s="4" t="inlineStr"/>
       <c r="I59" s="4" t="inlineStr">
         <is>
-          <t>https://www.galvaoesilva.com/escritorio-de-advocacia-em-porto-velho-ro/</t>
+          <t>https://hospitalsamar.com.br/</t>
         </is>
       </c>
       <c r="J59" s="4" t="inlineStr">
         <is>
-          <t>CNPJ 22.889.244/0001-00 | OAB/DF 2609/15</t>
+          <t>0800 033 0393 | Porto Velho: Av. Calama, 2585, Liberdade | Cacoal: Av. Sao Paulo, 2326, Centro | JI-PARANA: R. Padre Adolfo Rhol, 1267, Casa Preta</t>
         </is>
       </c>
       <c r="K59" s="4" t="inlineStr">
         <is>
-          <t>Banca nacional com unidade em Porto Velho. Tem pagina BANCO DE TALENTOS - caminho de entrada.</t>
+          <t>Maior rede hospitalar de RO. Tem pagina TRABALHE CONOSCO e pagina PARCEIROS.</t>
         </is>
       </c>
       <c r="L59" s="4" t="inlineStr">
@@ -3968,12 +3968,12 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>Rede Hospitalar Samar</t>
+          <t>Voo Transportes</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Porto Velho</t>
+          <t>Ji-Paraná</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
@@ -3988,28 +3988,28 @@
       </c>
       <c r="F60" s="6" t="inlineStr">
         <is>
-          <t>0800 033 0393</t>
+          <t>(69) 9908-1757</t>
         </is>
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
-          <t>Contencioso de saude e trabalhista</t>
+          <t>Assessoria trabalhista e civel</t>
         </is>
       </c>
       <c r="H60" s="4" t="inlineStr"/>
       <c r="I60" s="4" t="inlineStr">
         <is>
-          <t>https://hospitalsamar.com.br/</t>
+          <t>https://www.vootransportes.com.br/</t>
         </is>
       </c>
       <c r="J60" s="4" t="inlineStr">
         <is>
-          <t>0800 033 0393 | Porto Velho: Av. Calama, 2585, Liberdade | Cacoal: Av. Sao Paulo, 2326, Centro | JI-PARANA: R. Padre Adolfo Rhol, 1267, Casa Preta</t>
+          <t>Unidades: Ji-Parana (69) 9908-1757, Pimenta Bueno (69) 99226-5040, Porto Velho (69) 9983-0113, Rio Branco (68) 9232-9905, Guarulhos/SP (11) 2446-4276</t>
         </is>
       </c>
       <c r="K60" s="4" t="inlineStr">
         <is>
-          <t>Maior rede hospitalar de RO. Tem pagina TRABALHE CONOSCO e pagina PARCEIROS.</t>
+          <t>Unidade em Ji-Parana desde a fundacao. Sem e-mail no site.</t>
         </is>
       </c>
       <c r="L60" s="4" t="inlineStr">
@@ -4026,12 +4026,12 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Voo Transportes</t>
+          <t>Supermercados Irmãos Gonçalves</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Ji-Paraná</t>
+          <t>Jaru</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
@@ -4039,35 +4039,35 @@
           <t>RO</t>
         </is>
       </c>
-      <c r="E61" s="7" t="inlineStr">
-        <is>
-          <t>TELEFONE</t>
+      <c r="E61" s="10" t="inlineStr">
+        <is>
+          <t>FORMULARIO</t>
         </is>
       </c>
       <c r="F61" s="6" t="inlineStr">
         <is>
-          <t>(69) 9908-1757</t>
+          <t>https://www.irmaosgoncalves.com.br/</t>
         </is>
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
-          <t>Assessoria trabalhista e civel</t>
+          <t>Assessoria trabalhista e consumerista</t>
         </is>
       </c>
       <c r="H61" s="4" t="inlineStr"/>
       <c r="I61" s="4" t="inlineStr">
         <is>
-          <t>https://www.vootransportes.com.br/</t>
+          <t>https://www.irmaosgoncalves.com.br/</t>
         </is>
       </c>
       <c r="J61" s="4" t="inlineStr">
         <is>
-          <t>Unidades: Ji-Parana (69) 9908-1757, Pimenta Bueno (69) 99226-5040, Porto Velho (69) 9983-0113, Rio Branco (68) 9232-9905, Guarulhos/SP (11) 2446-4276</t>
+          <t>Paginas: Central de Atendimento, FALE CONOSCO e TRABALHE CONOSCO | Tem cartao proprio (IG Card)</t>
         </is>
       </c>
       <c r="K61" s="4" t="inlineStr">
         <is>
-          <t>Unidade em Ji-Parana desde a fundacao. Sem e-mail no site.</t>
+          <t>3a maior empresa de Rondonia por faturamento (R$ 7,2 bi). O IG Card e credito proprio, o que soma contencioso bancario e de cobranca ao trabalhista e consumerista do varejo.</t>
         </is>
       </c>
       <c r="L61" s="4" t="inlineStr">
@@ -4077,55 +4077,55 @@
       </c>
     </row>
     <row r="62" ht="62" customHeight="1">
-      <c r="A62" s="7" t="inlineStr">
-        <is>
-          <t>3. RONDÔNIA — cliente ou parceiro local</t>
+      <c r="A62" s="10" t="inlineStr">
+        <is>
+          <t>4. BANCA NACIONAL — ofereça correspondência em RO</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>Supermercados Irmãos Gonçalves</t>
+          <t>Bueno Brandão Advocacia</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>Jaru</t>
+          <t>São Paulo</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>RO</t>
-        </is>
-      </c>
-      <c r="E62" s="10" t="inlineStr">
-        <is>
-          <t>FORMULARIO</t>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>E-MAIL</t>
         </is>
       </c>
       <c r="F62" s="6" t="inlineStr">
         <is>
-          <t>https://www.irmaosgoncalves.com.br/</t>
+          <t>contato@buenobrandao.adv.br</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr">
         <is>
-          <t>Assessoria trabalhista e consumerista</t>
+          <t>Correspondencia em saude nas comarcas de RO</t>
         </is>
       </c>
       <c r="H62" s="4" t="inlineStr"/>
       <c r="I62" s="4" t="inlineStr">
         <is>
-          <t>https://www.irmaosgoncalves.com.br/</t>
+          <t>https://www.buenobrandao.adv.br/</t>
         </is>
       </c>
       <c r="J62" s="4" t="inlineStr">
         <is>
-          <t>Paginas: Central de Atendimento, FALE CONOSCO e TRABALHE CONOSCO | Tem cartao proprio (IG Card)</t>
+          <t>Tel (11) 3266-2067 | Alameda Casa Branca, 35, Cj. 510, Jd. Paulista, Sao Paulo/SP</t>
         </is>
       </c>
       <c r="K62" s="4" t="inlineStr">
         <is>
-          <t>3a maior empresa de Rondonia por faturamento (R$ 7,2 bi). O IG Card e credito proprio, o que soma contencioso bancario e de cobranca ao trabalhista e consumerista do varejo.</t>
+          <t>Especializada em Direito Medico e da Saude com atuacao em todo o territorio nacional.</t>
         </is>
       </c>
       <c r="L62" s="4" t="inlineStr">
@@ -4142,17 +4142,17 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>Bueno Brandão Advocacia</t>
+          <t>CMP Prev Advocacia</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>São Paulo</t>
+          <t>Florianópolis</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -4162,28 +4162,28 @@
       </c>
       <c r="F63" s="6" t="inlineStr">
         <is>
-          <t>contato@buenobrandao.adv.br</t>
+          <t>cmpprev@cmpprev.com.br</t>
         </is>
       </c>
       <c r="G63" s="4" t="inlineStr">
         <is>
-          <t>Correspondencia em saude nas comarcas de RO</t>
+          <t>Correspondencia previdenciaria em RO</t>
         </is>
       </c>
       <c r="H63" s="4" t="inlineStr"/>
       <c r="I63" s="4" t="inlineStr">
         <is>
-          <t>https://www.buenobrandao.adv.br/</t>
+          <t>https://cmpprev.com.br/</t>
         </is>
       </c>
       <c r="J63" s="4" t="inlineStr">
         <is>
-          <t>Tel (11) 3266-2067 | Alameda Casa Branca, 35, Cj. 510, Jd. Paulista, Sao Paulo/SP</t>
+          <t>0800 025 5009 (Juridico) | (48) 3025-5008 | WhatsApp (48) 7602-0501 | R. Jeronimo Coelho, 170, sala 1001, Centro, Florianopolis/SC</t>
         </is>
       </c>
       <c r="K63" s="4" t="inlineStr">
         <is>
-          <t>Especializada em Direito Medico e da Saude com atuacao em todo o territorio nacional.</t>
+          <t>ATENDE SEGURADOS DO INSS EM TODO O BRASIL, +25.000 casos. Escritorio oficial do SIMESC. Atuacao nacional sem estrutura local = precisam de correspondente para pericias e audiencias no JEF.</t>
         </is>
       </c>
       <c r="L63" s="4" t="inlineStr">
@@ -4200,17 +4200,17 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>CMP Prev Advocacia</t>
+          <t>Campanella Advocacia</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>Florianópolis</t>
+          <t>São Caetano do Sul</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -4220,28 +4220,28 @@
       </c>
       <c r="F64" s="6" t="inlineStr">
         <is>
-          <t>cmpprev@cmpprev.com.br</t>
+          <t>contato@campanellaadvocacia.com.br</t>
         </is>
       </c>
       <c r="G64" s="4" t="inlineStr">
         <is>
-          <t>Correspondencia previdenciaria em RO</t>
+          <t>Correspondencia em saude nas comarcas de RO</t>
         </is>
       </c>
       <c r="H64" s="4" t="inlineStr"/>
       <c r="I64" s="4" t="inlineStr">
         <is>
-          <t>https://cmpprev.com.br/</t>
+          <t>https://campanellaadvocacia.com.br/</t>
         </is>
       </c>
       <c r="J64" s="4" t="inlineStr">
         <is>
-          <t>0800 025 5009 (Juridico) | (48) 3025-5008 | WhatsApp (48) 7602-0501 | R. Jeronimo Coelho, 170, sala 1001, Centro, Florianopolis/SC</t>
+          <t>WhatsApp (11) 98118-0334 | Tel (11) 4224-3769 / 2988-7681 | Rua Para, 139, Sala 304, Centro, Sao Caetano do Sul-SP</t>
         </is>
       </c>
       <c r="K64" s="4" t="inlineStr">
         <is>
-          <t>ATENDE SEGURADOS DO INSS EM TODO O BRASIL, +25.000 casos. Escritorio oficial do SIMESC. Atuacao nacional sem estrutura local = precisam de correspondente para pericias e audiencias no JEF.</t>
+          <t>10+ anos em direito da saude: revisao de mensalidade por faixa etaria, home care, reembolso, erro medico e MEDICAMENTO DE ALTO CUSTO contra o SUS - exatamente o seu repertorio.</t>
         </is>
       </c>
       <c r="L64" s="4" t="inlineStr">
@@ -4258,17 +4258,17 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>Campanella Advocacia</t>
+          <t>Cardoso Advocacia</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>São Caetano do Sul</t>
+          <t>Salvador</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -4278,7 +4278,7 @@
       </c>
       <c r="F65" s="6" t="inlineStr">
         <is>
-          <t>contato@campanellaadvocacia.com.br</t>
+          <t>contato@cardosoadvocacia.com.br</t>
         </is>
       </c>
       <c r="G65" s="4" t="inlineStr">
@@ -4289,17 +4289,17 @@
       <c r="H65" s="4" t="inlineStr"/>
       <c r="I65" s="4" t="inlineStr">
         <is>
-          <t>https://campanellaadvocacia.com.br/</t>
+          <t>https://cardosoadvocacia.com.br/</t>
         </is>
       </c>
       <c r="J65" s="4" t="inlineStr">
         <is>
-          <t>WhatsApp (11) 98118-0334 | Tel (11) 4224-3769 / 2988-7681 | Rua Para, 139, Sala 304, Centro, Sao Caetano do Sul-SP</t>
+          <t>Tel (71) 99695-0180 / (71) 3034-3159 | Sede Salvador/BA + unidade Pinheiros, Sao Paulo/SP | CNPJ 15.176.644/0001-02 | OAB/BA 2056/2011</t>
         </is>
       </c>
       <c r="K65" s="4" t="inlineStr">
         <is>
-          <t>10+ anos em direito da saude: revisao de mensalidade por faixa etaria, home care, reembolso, erro medico e MEDICAMENTO DE ALTO CUSTO contra o SUS - exatamente o seu repertorio.</t>
+          <t>Texto do site: "ATUAMOS NO BRASIL INTEIRO - estamos presentes em MAIS DE 21 ESTADOS". Planos de saude. Operacao nacional a distancia precisa de gente nas comarcas.</t>
         </is>
       </c>
       <c r="L65" s="4" t="inlineStr">
@@ -4316,17 +4316,17 @@
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>Cardoso Advocacia</t>
+          <t>Delgado Azevedo Advogados</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>Salvador</t>
+          <t>Brasília</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>DF</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -4336,7 +4336,7 @@
       </c>
       <c r="F66" s="6" t="inlineStr">
         <is>
-          <t>contato@cardosoadvocacia.com.br</t>
+          <t>contato@delgadoazevedo.com.br</t>
         </is>
       </c>
       <c r="G66" s="4" t="inlineStr">
@@ -4347,17 +4347,17 @@
       <c r="H66" s="4" t="inlineStr"/>
       <c r="I66" s="4" t="inlineStr">
         <is>
-          <t>https://cardosoadvocacia.com.br/</t>
+          <t>https://www.delgadoazevedo.com.br/</t>
         </is>
       </c>
       <c r="J66" s="4" t="inlineStr">
         <is>
-          <t>Tel (71) 99695-0180 / (71) 3034-3159 | Sede Salvador/BA + unidade Pinheiros, Sao Paulo/SP | CNPJ 15.176.644/0001-02 | OAB/BA 2056/2011</t>
+          <t>Tel (61) 99955-8009 | Gabriel Espindola de Souza OAB-DF 71.982</t>
         </is>
       </c>
       <c r="K66" s="4" t="inlineStr">
         <is>
-          <t>Texto do site: "ATUAMOS NO BRASIL INTEIRO - estamos presentes em MAIS DE 21 ESTADOS". Planos de saude. Operacao nacional a distancia precisa de gente nas comarcas.</t>
+          <t>Declaram ATUACAO NACIONAL e atendimento 24 horas, em todos os tribunais do Brasil. Liminar, home care, negativa de medicamento e internacao - teses que voce ja domina.</t>
         </is>
       </c>
       <c r="L66" s="4" t="inlineStr">
@@ -4374,17 +4374,17 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>Delgado Azevedo Advogados</t>
+          <t>GAMAA - Advocacia de Bancos &amp; Empresas</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>Brasília</t>
+          <t>Belo Horizonte</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>DF</t>
+          <t>MG</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -4394,28 +4394,28 @@
       </c>
       <c r="F67" s="6" t="inlineStr">
         <is>
-          <t>contato@delgadoazevedo.com.br</t>
+          <t>contato@gamaa.com.br</t>
         </is>
       </c>
       <c r="G67" s="4" t="inlineStr">
         <is>
-          <t>Correspondencia em saude nas comarcas de RO</t>
+          <t>Parceria e correspondencia em RO</t>
         </is>
       </c>
       <c r="H67" s="4" t="inlineStr"/>
       <c r="I67" s="4" t="inlineStr">
         <is>
-          <t>https://www.delgadoazevedo.com.br/</t>
+          <t>https://gamaa.com.br/</t>
         </is>
       </c>
       <c r="J67" s="4" t="inlineStr">
         <is>
-          <t>Tel (61) 99955-8009 | Gabriel Espindola de Souza OAB-DF 71.982</t>
+          <t>Tel (31) 3274-9120 | R. Sao Paulo, 1071, 10o andar, Bloco B, Centro, BH/MG | Gilberto Miranda (proprietario)</t>
         </is>
       </c>
       <c r="K67" s="4" t="inlineStr">
         <is>
-          <t>Declaram ATUACAO NACIONAL e atendimento 24 horas, em todos os tribunais do Brasil. Liminar, home care, negativa de medicamento e internacao - teses que voce ja domina.</t>
+          <t>TEXTO DO PROPRIO SITE: "firmou parcerias com diversos escritorios de advogados do pais e POSSUI VARIOS CORRESPONDENTES no interior do estado de Minas Gerais". Ja usam o modelo. Clientes: Santander, Azul, BRF, Danone, Pernambucanas, Leroy Merlin. Tem pagina PARCEIROS.</t>
         </is>
       </c>
       <c r="L67" s="4" t="inlineStr">
@@ -4432,17 +4432,17 @@
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>GAMAA - Advocacia de Bancos &amp; Empresas</t>
+          <t>Gantus Advogados Associados</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>Belo Horizonte</t>
+          <t>São Paulo</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>MG</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -4452,28 +4452,28 @@
       </c>
       <c r="F68" s="6" t="inlineStr">
         <is>
-          <t>contato@gamaa.com.br</t>
+          <t>contato@gantusadvogados.com.br</t>
         </is>
       </c>
       <c r="G68" s="4" t="inlineStr">
         <is>
-          <t>Parceria e correspondencia em RO</t>
+          <t>Correspondencia para a carteira de massa em RO</t>
         </is>
       </c>
       <c r="H68" s="4" t="inlineStr"/>
       <c r="I68" s="4" t="inlineStr">
         <is>
-          <t>https://gamaa.com.br/</t>
+          <t>https://gantusadvogados.com.br/</t>
         </is>
       </c>
       <c r="J68" s="4" t="inlineStr">
         <is>
-          <t>Tel (31) 3274-9120 | R. Sao Paulo, 1071, 10o andar, Bloco B, Centro, BH/MG | Gilberto Miranda (proprietario)</t>
+          <t>Tel (11) 94924-8141 / (11) 3813-5211 | Alameda Joaquim Eugenio de Lima, 696, Jardins, Sao Paulo/SP | Filial em Brasilia/DF | Fundador: Guilherme Miguel Gantus</t>
         </is>
       </c>
       <c r="K68" s="4" t="inlineStr">
         <is>
-          <t>TEXTO DO PROPRIO SITE: "firmou parcerias com diversos escritorios de advogados do pais e POSSUI VARIOS CORRESPONDENTES no interior do estado de Minas Gerais". Ja usam o modelo. Clientes: Santander, Azul, BRF, Danone, Pernambucanas, Leroy Merlin. Tem pagina PARCEIROS.</t>
+          <t>Area declarada de CONTENCIOSO DE MASSA e atuacao em TODO O TERRITORIO NACIONAL com apenas duas sedes (SP e DF). Dependem de correspondente fora do eixo.</t>
         </is>
       </c>
       <c r="L68" s="4" t="inlineStr">
@@ -4490,17 +4490,17 @@
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>Gantus Advogados Associados</t>
+          <t>Gilmar Araujo da Costa Advocacia</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>São Paulo</t>
+          <t>Manaus</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>AM</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -4510,28 +4510,28 @@
       </c>
       <c r="F69" s="6" t="inlineStr">
         <is>
-          <t>contato@gantusadvogados.com.br</t>
+          <t>gac.advogado89@gmail.com</t>
         </is>
       </c>
       <c r="G69" s="4" t="inlineStr">
         <is>
-          <t>Correspondencia para a carteira de massa em RO</t>
+          <t>Correspondencia em RO - consumidor e bancario</t>
         </is>
       </c>
       <c r="H69" s="4" t="inlineStr"/>
       <c r="I69" s="4" t="inlineStr">
         <is>
-          <t>https://gantusadvogados.com.br/</t>
+          <t>https://gilmararaujoadvocacia.com.br/</t>
         </is>
       </c>
       <c r="J69" s="4" t="inlineStr">
         <is>
-          <t>Tel (11) 94924-8141 / (11) 3813-5211 | Alameda Joaquim Eugenio de Lima, 696, Jardins, Sao Paulo/SP | Filial em Brasilia/DF | Fundador: Guilherme Miguel Gantus</t>
+          <t>Tel (92) 98441-1276 | R. Rio Tarauaca, 36, Nossa Sra. das Gracas, Manaus-AM | CNPJ 46.366.996/0001-54</t>
         </is>
       </c>
       <c r="K69" s="4" t="inlineStr">
         <is>
-          <t>Area declarada de CONTENCIOSO DE MASSA e atuacao em TODO O TERRITORIO NACIONAL com apenas duas sedes (SP e DF). Dependem de correspondente fora do eixo.</t>
+          <t>Atuacao declarada EM TODO O BRASIL em consumidor e bancario: cartao RMC, consignado nao solicitado, juros abusivos, negativacao indevida. Mesmas teses que voce domina. Regiao Norte.</t>
         </is>
       </c>
       <c r="L69" s="4" t="inlineStr">
@@ -4548,17 +4548,17 @@
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>Gilmar Araujo da Costa Advocacia</t>
+          <t>LDCM Advogados</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>Manaus</t>
+          <t>Rio de Janeiro</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>AM</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
@@ -4568,28 +4568,28 @@
       </c>
       <c r="F70" s="6" t="inlineStr">
         <is>
-          <t>gac.advogado89@gmail.com</t>
+          <t>contato@ldcm.com.br</t>
         </is>
       </c>
       <c r="G70" s="4" t="inlineStr">
         <is>
-          <t>Correspondencia em RO - consumidor e bancario</t>
+          <t>Correspondencia para carteiras de bancario, telecom e varejo</t>
         </is>
       </c>
       <c r="H70" s="4" t="inlineStr"/>
       <c r="I70" s="4" t="inlineStr">
         <is>
-          <t>https://gilmararaujoadvocacia.com.br/</t>
+          <t>https://www.ldcm.com.br/</t>
         </is>
       </c>
       <c r="J70" s="4" t="inlineStr">
         <is>
-          <t>Tel (92) 98441-1276 | R. Rio Tarauaca, 36, Nossa Sra. das Gracas, Manaus-AM | CNPJ 46.366.996/0001-54</t>
+          <t>Tel RJ +55 21 3500-3990 | SP +55 11 4380-8626 | Av. Epitacio Pessoa, 1.274, Ipanema, RJ | Av. Brig. Faria Lima, 4.300, Vila Olimpia, SP | E-mail nominal publicado: bruno.barreto@ldcm.com.br</t>
         </is>
       </c>
       <c r="K70" s="4" t="inlineStr">
         <is>
-          <t>Atuacao declarada EM TODO O BRASIL em consumidor e bancario: cartao RMC, consignado nao solicitado, juros abusivos, negativacao indevida. Mesmas teses que voce domina. Regiao Norte.</t>
+          <t>Boutique de disputas com carteira declarada em bancario, telecomunicacoes e varejo - os tres setores de maior contencioso de massa. So duas pracas.</t>
         </is>
       </c>
       <c r="L70" s="4" t="inlineStr">
@@ -4606,17 +4606,17 @@
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>LDCM Advogados</t>
+          <t>Marcelo Tostes Advogados - contato geral</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>Rio de Janeiro</t>
+          <t>Belo Horizonte</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>RJ</t>
+          <t>MG</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
@@ -4626,28 +4626,28 @@
       </c>
       <c r="F71" s="6" t="inlineStr">
         <is>
-          <t>contato@ldcm.com.br</t>
+          <t>contato@mtostes.com.br</t>
         </is>
       </c>
       <c r="G71" s="4" t="inlineStr">
         <is>
-          <t>Correspondencia para carteiras de bancario, telecom e varejo</t>
+          <t>Correspondencia em RO / candidatura</t>
         </is>
       </c>
       <c r="H71" s="4" t="inlineStr"/>
       <c r="I71" s="4" t="inlineStr">
         <is>
-          <t>https://www.ldcm.com.br/</t>
+          <t>https://mtostes.com.br/</t>
         </is>
       </c>
       <c r="J71" s="4" t="inlineStr">
         <is>
-          <t>Tel RJ +55 21 3500-3990 | SP +55 11 4380-8626 | Av. Epitacio Pessoa, 1.274, Ipanema, RJ | Av. Brig. Faria Lima, 4.300, Vila Olimpia, SP | E-mail nominal publicado: bruno.barreto@ldcm.com.br</t>
+          <t>Unidades e telefones: SP (11) 4837-3400, BH (31) 4501-4100, Porto Alegre (51) 3103-4901, Vitoria (27) 3345-1999, Brasilia (61) 3225-4774, Rio de Janeiro, Florianopolis</t>
         </is>
       </c>
       <c r="K71" s="4" t="inlineStr">
         <is>
-          <t>Boutique de disputas com carteira declarada em bancario, telecomunicacoes e varejo - os tres setores de maior contencioso de massa. So duas pracas.</t>
+          <t>SEGUNDO E-MAIL da banca (o outro e recrutamento@mtostes.com.br). Area declarada "Contencioso Escala" e "Service, Backoffice &amp; Gestao de Dados". Nenhuma unidade no Norte.</t>
         </is>
       </c>
       <c r="L71" s="4" t="inlineStr">
@@ -4664,17 +4664,17 @@
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>Marcelo Tostes Advogados - contato geral</t>
+          <t>Nelson Wilians Advogados (NWADV) - fundador</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>Belo Horizonte</t>
+          <t>São Paulo</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>MG</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -4684,28 +4684,28 @@
       </c>
       <c r="F72" s="6" t="inlineStr">
         <is>
-          <t>contato@mtostes.com.br</t>
+          <t>nelson@nwadv.com.br</t>
         </is>
       </c>
       <c r="G72" s="4" t="inlineStr">
         <is>
-          <t>Correspondencia em RO / candidatura</t>
+          <t>Correspondencia / associacao - maior banca do pais</t>
         </is>
       </c>
       <c r="H72" s="4" t="inlineStr"/>
       <c r="I72" s="4" t="inlineStr">
         <is>
-          <t>https://mtostes.com.br/</t>
+          <t>https://www.nwadv.com.br/</t>
         </is>
       </c>
       <c r="J72" s="4" t="inlineStr">
         <is>
-          <t>Unidades e telefones: SP (11) 4837-3400, BH (31) 4501-4100, Porto Alegre (51) 3103-4901, Vitoria (27) 3345-1999, Brasilia (61) 3225-4774, Rio de Janeiro, Florianopolis</t>
+          <t>Tel SP (11) 3330-2299 | Unidades com telefone proprio em TODOS os estados, incluindo RONDONIA | Manaus (92) 3659-3954, Rio Branco (68) 3222-8576, Macapa (96) 3224-1169, Brasilia (61) 3106-2000</t>
         </is>
       </c>
       <c r="K72" s="4" t="inlineStr">
         <is>
-          <t>SEGUNDO E-MAIL da banca (o outro e recrutamento@mtostes.com.br). Area declarada "Contencioso Escala" e "Service, Backoffice &amp; Gestao de Dados". Nenhuma unidade no Norte.</t>
+          <t>E-MAIL DO PROPRIO FUNDADOR publicado no site. Declaram PRESENCA FISICA EM TODOS OS ESTADOS BRASILEIROS. Ja tem unidade em Porto Velho - o encaixe aqui e cobrir as comarcas do INTERIOR de RO, onde a unidade da capital nao chega.</t>
         </is>
       </c>
       <c r="L72" s="4" t="inlineStr">
@@ -4722,7 +4722,7 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>Nelson Wilians Advogados (NWADV) - fundador</t>
+          <t>Parra Advogados</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
@@ -4742,28 +4742,28 @@
       </c>
       <c r="F73" s="6" t="inlineStr">
         <is>
-          <t>nelson@nwadv.com.br</t>
+          <t>contato@parraadvogados.com.br</t>
         </is>
       </c>
       <c r="G73" s="4" t="inlineStr">
         <is>
-          <t>Correspondencia / associacao - maior banca do pais</t>
+          <t>Correspondencia em saude e securitario em RO</t>
         </is>
       </c>
       <c r="H73" s="4" t="inlineStr"/>
       <c r="I73" s="4" t="inlineStr">
         <is>
-          <t>https://www.nwadv.com.br/</t>
+          <t>https://www.parraadvogados.com.br/</t>
         </is>
       </c>
       <c r="J73" s="4" t="inlineStr">
         <is>
-          <t>Tel SP (11) 3330-2299 | Unidades com telefone proprio em TODOS os estados, incluindo RONDONIA | Manaus (92) 3659-3954, Rio Branco (68) 3222-8576, Macapa (96) 3224-1169, Brasilia (61) 3106-2000</t>
+          <t>Tel (11) 2092-8728 / (11) 94529-1615 | R. Nova Jerusalem, 740, sala 1, Chacara Santo Antonio, Sao Paulo/SP | OAB/SP 18.155</t>
         </is>
       </c>
       <c r="K73" s="4" t="inlineStr">
         <is>
-          <t>E-MAIL DO PROPRIO FUNDADOR publicado no site. Declaram PRESENCA FISICA EM TODOS OS ESTADOS BRASILEIROS. Ja tem unidade em Porto Velho - o encaixe aqui e cobrir as comarcas do INTERIOR de RO, onde a unidade da capital nao chega.</t>
+          <t>ENCAIXE PERFEITO: o site diz que prestam servico "com atendimento em TODO BRASIL, presencial ou virtual, MEDIANTE CONTRATACAO POR SERVICO ou assessoria mensal". E o modelo de correspondente descrito com outras palavras. Especialistas em liminares contra planos de saude - sua area.</t>
         </is>
       </c>
       <c r="L73" s="4" t="inlineStr">
@@ -4780,7 +4780,7 @@
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>Parra Advogados</t>
+          <t>R. Barreto Advogados</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
@@ -4800,28 +4800,28 @@
       </c>
       <c r="F74" s="6" t="inlineStr">
         <is>
-          <t>contato@parraadvogados.com.br</t>
+          <t>rbarreto@rbarreto.adv.br</t>
         </is>
       </c>
       <c r="G74" s="4" t="inlineStr">
         <is>
-          <t>Correspondencia em saude e securitario em RO</t>
+          <t>Correspondencia e audiencias em RO</t>
         </is>
       </c>
       <c r="H74" s="4" t="inlineStr"/>
       <c r="I74" s="4" t="inlineStr">
         <is>
-          <t>https://www.parraadvogados.com.br/</t>
+          <t>https://www.rbarreto.adv.br/</t>
         </is>
       </c>
       <c r="J74" s="4" t="inlineStr">
         <is>
-          <t>Tel (11) 2092-8728 / (11) 94529-1615 | R. Nova Jerusalem, 740, sala 1, Chacara Santo Antonio, Sao Paulo/SP | OAB/SP 18.155</t>
+          <t>Tel (11) 3044-2293 | Av. Nove de Julho, 4254, Jardim Paulista, Sao Paulo/SP</t>
         </is>
       </c>
       <c r="K74" s="4" t="inlineStr">
         <is>
-          <t>ENCAIXE PERFEITO: o site diz que prestam servico "com atendimento em TODO BRASIL, presencial ou virtual, MEDIANTE CONTRATACAO POR SERVICO ou assessoria mensal". E o modelo de correspondente descrito com outras palavras. Especialistas em liminares contra planos de saude - sua area.</t>
+          <t>Numeros do proprio site: +22.000 acoes contrarias, +4.000 processos de recuperacao de credito, R$ 80 milhoes recuperados. ATENDEM TODO O BRASIL DE FORMA REMOTA - precisam de gente em campo nas comarcas.</t>
         </is>
       </c>
       <c r="L74" s="4" t="inlineStr">
@@ -4838,17 +4838,17 @@
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>R. Barreto Advogados</t>
+          <t>Ribeiro &amp; Feitoza Advogados</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>São Paulo</t>
+          <t>Manaus</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>AM</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -4858,28 +4858,28 @@
       </c>
       <c r="F75" s="6" t="inlineStr">
         <is>
-          <t>rbarreto@rbarreto.adv.br</t>
+          <t>contato@ribeiroefeitozaadvogados.com</t>
         </is>
       </c>
       <c r="G75" s="4" t="inlineStr">
         <is>
-          <t>Correspondencia e audiencias em RO</t>
+          <t>Parceria e correspondencia na regiao Norte</t>
         </is>
       </c>
       <c r="H75" s="4" t="inlineStr"/>
       <c r="I75" s="4" t="inlineStr">
         <is>
-          <t>https://www.rbarreto.adv.br/</t>
+          <t>https://ribeiroefeitozaadvogados.com.br/</t>
         </is>
       </c>
       <c r="J75" s="4" t="inlineStr">
         <is>
-          <t>Tel (11) 3044-2293 | Av. Nove de Julho, 4254, Jardim Paulista, Sao Paulo/SP</t>
+          <t>Tel +55 92 99147-9179 | Avenida Getulio Vargas, 1222, Centro, Manaus/AM</t>
         </is>
       </c>
       <c r="K75" s="4" t="inlineStr">
         <is>
-          <t>Numeros do proprio site: +22.000 acoes contrarias, +4.000 processos de recuperacao de credito, R$ 80 milhoes recuperados. ATENDEM TODO O BRASIL DE FORMA REMOTA - precisam de gente em campo nas comarcas.</t>
+          <t>12 anos, referencia no Amazonas. Atuam em consumidor, bancario, licitacoes e ESG. Regiao Norte - logistica e cultura processual iguais as de RO.</t>
         </is>
       </c>
       <c r="L75" s="4" t="inlineStr">
@@ -4896,17 +4896,17 @@
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>Ribeiro &amp; Feitoza Advogados</t>
+          <t>SSantos Advogados</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>Manaus</t>
+          <t>Curitiba</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>AM</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
@@ -4916,28 +4916,28 @@
       </c>
       <c r="F76" s="6" t="inlineStr">
         <is>
-          <t>contato@ribeiroefeitozaadvogados.com</t>
+          <t>advocacia@ssantos.adv.br</t>
         </is>
       </c>
       <c r="G76" s="4" t="inlineStr">
         <is>
-          <t>Parceria e correspondencia na regiao Norte</t>
+          <t>Correspondencia previdenciaria em RO</t>
         </is>
       </c>
       <c r="H76" s="4" t="inlineStr"/>
       <c r="I76" s="4" t="inlineStr">
         <is>
-          <t>https://ribeiroefeitozaadvogados.com.br/</t>
+          <t>https://ssantos.adv.br/</t>
         </is>
       </c>
       <c r="J76" s="4" t="inlineStr">
         <is>
-          <t>Tel +55 92 99147-9179 | Avenida Getulio Vargas, 1222, Centro, Manaus/AM</t>
+          <t>(41) 3023-1498 principal | (41) 98850-9639 comercial | Rua Emiliano Perneta, 680, 5o andar, Centro, Curitiba-PR</t>
         </is>
       </c>
       <c r="K76" s="4" t="inlineStr">
         <is>
-          <t>12 anos, referencia no Amazonas. Atuam em consumidor, bancario, licitacoes e ESG. Regiao Norte - logistica e cultura processual iguais as de RO.</t>
+          <t>Presenca fisica em 6 ESTADOS (PR, SP, ES, BA, SP-Santos) e parceiros estrategicos em outros. 23 anos em revisao de aposentadoria. Parceria com +10 associacoes de aposentados. Norte descoberto.</t>
         </is>
       </c>
       <c r="L76" s="4" t="inlineStr">
@@ -4954,17 +4954,17 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>SSantos Advogados</t>
+          <t>Tomás de Souza Sociedade de Advocacia</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>Curitiba</t>
+          <t>Brasília</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>DF</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -4974,28 +4974,28 @@
       </c>
       <c r="F77" s="6" t="inlineStr">
         <is>
-          <t>advocacia@ssantos.adv.br</t>
+          <t>tomasdesouzaadvogados@gmail.com</t>
         </is>
       </c>
       <c r="G77" s="4" t="inlineStr">
         <is>
-          <t>Correspondencia previdenciaria em RO</t>
+          <t>Entrar na rede de advogados associados</t>
         </is>
       </c>
       <c r="H77" s="4" t="inlineStr"/>
       <c r="I77" s="4" t="inlineStr">
         <is>
-          <t>https://ssantos.adv.br/</t>
+          <t>https://tomasdesouzaadvogados.com.br/</t>
         </is>
       </c>
       <c r="J77" s="4" t="inlineStr">
         <is>
-          <t>(41) 3023-1498 principal | (41) 98850-9639 comercial | Rua Emiliano Perneta, 680, 5o andar, Centro, Curitiba-PR</t>
+          <t>Tel (61) 99221-1401 | Sede: SMPW Q22, Cj 01, Lote 07, Casa B, Park Way, Brasilia/DF | Unidade: Rua 122, 216, Setor Sul, Goiania/GO</t>
         </is>
       </c>
       <c r="K77" s="4" t="inlineStr">
         <is>
-          <t>Presenca fisica em 6 ESTADOS (PR, SP, ES, BA, SP-Santos) e parceiros estrategicos em outros. 23 anos em revisao de aposentadoria. Parceria com +10 associacoes de aposentados. Norte descoberto.</t>
+          <t>TEXTO DO SITE: atuam "com o APOIO DE UMA REDE DE ADVOGADOS ASSOCIADOS". Ja operam no modelo. Atuacao em tribunais superiores e Justica Federal. So duas pracas.</t>
         </is>
       </c>
       <c r="L77" s="4" t="inlineStr">
@@ -5012,17 +5012,17 @@
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>Tomás de Souza Sociedade de Advocacia</t>
+          <t>Trajano Neto &amp; Paciornik Advogados (TNP)</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>Brasília</t>
+          <t>Curitiba</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>DF</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -5032,28 +5032,28 @@
       </c>
       <c r="F78" s="6" t="inlineStr">
         <is>
-          <t>tomasdesouzaadvogados@gmail.com</t>
+          <t>contato@tnp.adv.br</t>
         </is>
       </c>
       <c r="G78" s="4" t="inlineStr">
         <is>
-          <t>Entrar na rede de advogados associados</t>
+          <t>Correspondencia na rede de coligados - comarcas de RO</t>
         </is>
       </c>
       <c r="H78" s="4" t="inlineStr"/>
       <c r="I78" s="4" t="inlineStr">
         <is>
-          <t>https://tomasdesouzaadvogados.com.br/</t>
+          <t>https://tnp.adv.br/novosite/gestao-do-contencioso-de-massa/</t>
         </is>
       </c>
       <c r="J78" s="4" t="inlineStr">
         <is>
-          <t>Tel (61) 99221-1401 | Sede: SMPW Q22, Cj 01, Lote 07, Casa B, Park Way, Brasilia/DF | Unidade: Rua 122, 216, Setor Sul, Goiania/GO</t>
+          <t>0800 575 0011 | +55 41 3075-5020 | Euripedes Garcez do Nascimento, 549, Ahu, Curitiba/PR</t>
         </is>
       </c>
       <c r="K78" s="4" t="inlineStr">
         <is>
-          <t>TEXTO DO SITE: atuam "com o APOIO DE UMA REDE DE ADVOGADOS ASSOCIADOS". Ja operam no modelo. Atuacao em tribunais superiores e Justica Federal. So duas pracas.</t>
+          <t>ALVO NUMERO 1 DE CORRESPONDENCIA: area declarada de GESTAO DO CONTENCIOSO DE MASSA operando com "REDE DE COLIGADOS EM TODO BRASIL". Unidades: Brasilia, Natal, Sao Luis, Guarapuava, Florianopolis, Sao Paulo, Fortaleza - NENHUMA NO NORTE. Rondonia e buraco na malha deles.</t>
         </is>
       </c>
       <c r="L78" s="4" t="inlineStr">
@@ -5070,17 +5070,17 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>Trajano Neto &amp; Paciornik Advogados (TNP)</t>
+          <t>Ultreia Contábil</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>Curitiba</t>
+          <t>Brasília</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>DF</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -5090,28 +5090,28 @@
       </c>
       <c r="F79" s="6" t="inlineStr">
         <is>
-          <t>contato@tnp.adv.br</t>
+          <t>assessoria@ultreiacontabil.com.br</t>
         </is>
       </c>
       <c r="G79" s="4" t="inlineStr">
         <is>
-          <t>Correspondencia na rede de coligados - comarcas de RO</t>
+          <t>Parceria contabil-juridica</t>
         </is>
       </c>
       <c r="H79" s="4" t="inlineStr"/>
       <c r="I79" s="4" t="inlineStr">
         <is>
-          <t>https://tnp.adv.br/novosite/gestao-do-contencioso-de-massa/</t>
+          <t>https://ultreiacontabil.com.br/</t>
         </is>
       </c>
       <c r="J79" s="4" t="inlineStr">
         <is>
-          <t>0800 575 0011 | +55 41 3075-5020 | Euripedes Garcez do Nascimento, 549, Ahu, Curitiba/PR</t>
+          <t>Tel (61) 99694-5756</t>
         </is>
       </c>
       <c r="K79" s="4" t="inlineStr">
         <is>
-          <t>ALVO NUMERO 1 DE CORRESPONDENCIA: area declarada de GESTAO DO CONTENCIOSO DE MASSA operando com "REDE DE COLIGADOS EM TODO BRASIL". Unidades: Brasilia, Natal, Sao Luis, Guarapuava, Florianopolis, Sao Paulo, Fortaleza - NENHUMA NO NORTE. Rondonia e buraco na malha deles.</t>
+          <t>ATENDE ADVOGADOS como especialidade declarada, e faz Planejamento e Recuperacao Tributaria - parceria natural na sua area tributaria.</t>
         </is>
       </c>
       <c r="L79" s="4" t="inlineStr">
@@ -5128,48 +5128,48 @@
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>Ultreia Contábil</t>
+          <t>Amil</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>Brasília</t>
+          <t>São Paulo</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>DF</t>
-        </is>
-      </c>
-      <c r="E80" s="5" t="inlineStr">
-        <is>
-          <t>E-MAIL</t>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E80" s="7" t="inlineStr">
+        <is>
+          <t>TELEFONE</t>
         </is>
       </c>
       <c r="F80" s="6" t="inlineStr">
         <is>
-          <t>assessoria@ultreiacontabil.com.br</t>
+          <t>0800 721 1094</t>
         </is>
       </c>
       <c r="G80" s="4" t="inlineStr">
         <is>
-          <t>Parceria contabil-juridica</t>
+          <t>Contencioso de saude suplementar</t>
         </is>
       </c>
       <c r="H80" s="4" t="inlineStr"/>
       <c r="I80" s="4" t="inlineStr">
         <is>
-          <t>https://ultreiacontabil.com.br/</t>
+          <t>https://www.amil.com.br/</t>
         </is>
       </c>
       <c r="J80" s="4" t="inlineStr">
         <is>
-          <t>Tel (61) 99694-5756</t>
+          <t>Ouvidoria: 3004-1094 (capitais) e 0800 721 1094 (demais localidades) | Av. Dr. Chucri Zaidan, 1649, Ed. EZ Towers, Torre B, 23o andar, Sao Paulo/SP</t>
         </is>
       </c>
       <c r="K80" s="4" t="inlineStr">
         <is>
-          <t>ATENDE ADVOGADOS como especialidade declarada, e faz Planejamento e Recuperacao Tributaria - parceria natural na sua area tributaria.</t>
+          <t>Operadora que mais cresceu em marco de 2026. Carteira nacional com contencioso disperso.</t>
         </is>
       </c>
       <c r="L80" s="4" t="inlineStr">
@@ -5186,12 +5186,12 @@
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>Amil</t>
+          <t>Bocchi Advogados Associados</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>São Paulo</t>
+          <t>Ribeirão Preto</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
@@ -5206,28 +5206,28 @@
       </c>
       <c r="F81" s="6" t="inlineStr">
         <is>
-          <t>0800 721 1094</t>
+          <t>0800 000 3373</t>
         </is>
       </c>
       <c r="G81" s="4" t="inlineStr">
         <is>
-          <t>Contencioso de saude suplementar</t>
+          <t>Correspondencia previdenciaria em RO</t>
         </is>
       </c>
       <c r="H81" s="4" t="inlineStr"/>
       <c r="I81" s="4" t="inlineStr">
         <is>
-          <t>https://www.amil.com.br/</t>
+          <t>https://bocchiadvogados.com.br/</t>
         </is>
       </c>
       <c r="J81" s="4" t="inlineStr">
         <is>
-          <t>Ouvidoria: 3004-1094 (capitais) e 0800 721 1094 (demais localidades) | Av. Dr. Chucri Zaidan, 1649, Ed. EZ Towers, Torre B, 23o andar, Sao Paulo/SP</t>
+          <t>Rua Amador Bueno, 800, Ribeirao Preto/SP</t>
         </is>
       </c>
       <c r="K81" s="4" t="inlineStr">
         <is>
-          <t>Operadora que mais cresceu em marco de 2026. Carteira nacional com contencioso disperso.</t>
+          <t>50+ anos em previdenciario, trabalhista e civel. Texto do site: "fornecemos servicos juridicos para clientes de TODO BRASIL E DO MUNDO". Uma sede so - dependem de apoio local.</t>
         </is>
       </c>
       <c r="L81" s="4" t="inlineStr">
@@ -5244,17 +5244,17 @@
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>Bocchi Advogados Associados</t>
+          <t>Escobar Advogados - Programa de Parcerias</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>Ribeirão Preto</t>
+          <t>Goiânia</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="E82" s="7" t="inlineStr">
@@ -5264,28 +5264,28 @@
       </c>
       <c r="F82" s="6" t="inlineStr">
         <is>
-          <t>0800 000 3373</t>
+          <t>(62) 3280-9271</t>
         </is>
       </c>
       <c r="G82" s="4" t="inlineStr">
         <is>
-          <t>Correspondencia previdenciaria em RO</t>
+          <t>Programa de parcerias previdenciario</t>
         </is>
       </c>
       <c r="H82" s="4" t="inlineStr"/>
       <c r="I82" s="4" t="inlineStr">
         <is>
-          <t>https://bocchiadvogados.com.br/</t>
+          <t>https://escobaradvogados.com/parcerias/</t>
         </is>
       </c>
       <c r="J82" s="4" t="inlineStr">
         <is>
-          <t>Rua Amador Bueno, 800, Ribeirao Preto/SP</t>
+          <t>Responsavel: Dra. Ana Lara | Parceiro recebe relatorios mensais e reunioes trimestrais</t>
         </is>
       </c>
       <c r="K82" s="4" t="inlineStr">
         <is>
-          <t>50+ anos em previdenciario, trabalhista e civel. Texto do site: "fornecemos servicos juridicos para clientes de TODO BRASIL E DO MUNDO". Uma sede so - dependem de apoio local.</t>
+          <t>ATENCAO: 1a fase limitada a GOIAS, expansao nacional prevista para a 2a etapa. Vale registrar interesse agora para entrar na expansao. Foco em beneficios do INSS.</t>
         </is>
       </c>
       <c r="L82" s="4" t="inlineStr">
@@ -5302,17 +5302,17 @@
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>Escobar Advogados - Programa de Parcerias</t>
+          <t>Hapvida NotreDame Intermédica</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>Goiânia</t>
+          <t>Fortaleza</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>CE</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
@@ -5322,28 +5322,28 @@
       </c>
       <c r="F83" s="6" t="inlineStr">
         <is>
-          <t>(62) 3280-9271</t>
+          <t>0800 280 9130</t>
         </is>
       </c>
       <c r="G83" s="4" t="inlineStr">
         <is>
-          <t>Programa de parcerias previdenciario</t>
+          <t>Contencioso de saude suplementar</t>
         </is>
       </c>
       <c r="H83" s="4" t="inlineStr"/>
       <c r="I83" s="4" t="inlineStr">
         <is>
-          <t>https://escobaradvogados.com/parcerias/</t>
+          <t>https://www.hapvida.com.br/</t>
         </is>
       </c>
       <c r="J83" s="4" t="inlineStr">
         <is>
-          <t>Responsavel: Dra. Ana Lara | Parceiro recebe relatorios mensais e reunioes trimestrais</t>
+          <t>0800 280 9130 (Norte e Nordeste) | 0800 018 3456 (Sul, Sudeste e Centro-Oeste) | Av. Heraclito Graca, 406, Centro, Fortaleza/CE | CNPJ 44.649.812/0001-38 | Tem TRABALHE CONOSCO e CANAL DE DENUNCIAS</t>
         </is>
       </c>
       <c r="K83" s="4" t="inlineStr">
         <is>
-          <t>ATENCAO: 1a fase limitada a GOIAS, expansao nacional prevista para a 2a etapa. Vale registrar interesse agora para entrar na expansao. Foco em beneficios do INSS.</t>
+          <t>Lider nacional em saude suplementar (8,8 milhoes de usuarios). Repare que tem 0800 ESPECIFICO para Norte e Nordeste - a operacao no Norte e separada.</t>
         </is>
       </c>
       <c r="L83" s="4" t="inlineStr">
@@ -5360,17 +5360,17 @@
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>Hapvida NotreDame Intermédica</t>
+          <t>Medina, Ribeiro &amp; Aguiar Advogados (MRA)</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>Fortaleza</t>
+          <t>Manaus</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>CE</t>
+          <t>AM</t>
         </is>
       </c>
       <c r="E84" s="7" t="inlineStr">
@@ -5380,28 +5380,28 @@
       </c>
       <c r="F84" s="6" t="inlineStr">
         <is>
-          <t>0800 280 9130</t>
+          <t>(92) 3242-0464</t>
         </is>
       </c>
       <c r="G84" s="4" t="inlineStr">
         <is>
-          <t>Contencioso de saude suplementar</t>
+          <t>Correspondencia na regiao Norte</t>
         </is>
       </c>
       <c r="H84" s="4" t="inlineStr"/>
       <c r="I84" s="4" t="inlineStr">
         <is>
-          <t>https://www.hapvida.com.br/</t>
+          <t>https://www.medinaeribeiro.com/</t>
         </is>
       </c>
       <c r="J84" s="4" t="inlineStr">
         <is>
-          <t>0800 280 9130 (Norte e Nordeste) | 0800 018 3456 (Sul, Sudeste e Centro-Oeste) | Av. Heraclito Graca, 406, Centro, Fortaleza/CE | CNPJ 44.649.812/0001-38 | Tem TRABALHE CONOSCO e CANAL DE DENUNCIAS</t>
+          <t>Forum Business Center, Sala 1702, Av. Andre Araujo, 97, Adrianopolis, Manaus/AM</t>
         </is>
       </c>
       <c r="K84" s="4" t="inlineStr">
         <is>
-          <t>Lider nacional em saude suplementar (8,8 milhoes de usuarios). Repare que tem 0800 ESPECIFICO para Norte e Nordeste - a operacao no Norte e separada.</t>
+          <t>Full service empresarial no Amazonas, consultivo e contencioso. Regiao Norte.</t>
         </is>
       </c>
       <c r="L84" s="4" t="inlineStr">
@@ -5418,17 +5418,17 @@
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>Medina, Ribeiro &amp; Aguiar Advogados (MRA)</t>
+          <t>RS Advocacia Previdenciária (Ribeiro e Silva)</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>Manaus</t>
+          <t>São Paulo</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>AM</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="E85" s="7" t="inlineStr">
@@ -5438,28 +5438,28 @@
       </c>
       <c r="F85" s="6" t="inlineStr">
         <is>
-          <t>(92) 3242-0464</t>
+          <t>(11) 4210-0217</t>
         </is>
       </c>
       <c r="G85" s="4" t="inlineStr">
         <is>
-          <t>Correspondencia na regiao Norte</t>
+          <t>Correspondencia previdenciaria em RO</t>
         </is>
       </c>
       <c r="H85" s="4" t="inlineStr"/>
       <c r="I85" s="4" t="inlineStr">
         <is>
-          <t>https://www.medinaeribeiro.com/</t>
+          <t>https://rsadvocaciaprevidenciaria.com.br/</t>
         </is>
       </c>
       <c r="J85" s="4" t="inlineStr">
         <is>
-          <t>Forum Business Center, Sala 1702, Av. Andre Araujo, 97, Adrianopolis, Manaus/AM</t>
+          <t>Telefone e WhatsApp (11) 4210-0217 | Av. Paulista, 1.106, 16o andar, Sala 1 | Unidade Mooca: Rua Ipanema, 80 | CNPJ 55.065.755/0001-10</t>
         </is>
       </c>
       <c r="K85" s="4" t="inlineStr">
         <is>
-          <t>Full service empresarial no Amazonas, consultivo e contencioso. Regiao Norte.</t>
+          <t>Atuam desde 2012 so em previdenciario, com CONSULTA ONLINE PARA TODO O BRASIL. BPC/LOAS, incapacidade, pensao por morte e revisoes - demandas do JEF de Ji-Parana.</t>
         </is>
       </c>
       <c r="L85" s="4" t="inlineStr">
@@ -5476,7 +5476,7 @@
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>RS Advocacia Previdenciária (Ribeiro e Silva)</t>
+          <t>SA Law Advogados</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
@@ -5496,28 +5496,28 @@
       </c>
       <c r="F86" s="6" t="inlineStr">
         <is>
-          <t>(11) 4210-0217</t>
+          <t>+55 (11) 3288-6060</t>
         </is>
       </c>
       <c r="G86" s="4" t="inlineStr">
         <is>
-          <t>Correspondencia previdenciaria em RO</t>
+          <t>Correspondencia e candidatura (pagina Careers)</t>
         </is>
       </c>
       <c r="H86" s="4" t="inlineStr"/>
       <c r="I86" s="4" t="inlineStr">
         <is>
-          <t>https://rsadvocaciaprevidenciaria.com.br/</t>
+          <t>https://salaw.com.br/</t>
         </is>
       </c>
       <c r="J86" s="4" t="inlineStr">
         <is>
-          <t>Telefone e WhatsApp (11) 4210-0217 | Av. Paulista, 1.106, 16o andar, Sala 1 | Unidade Mooca: Rua Ipanema, 80 | CNPJ 55.065.755/0001-10</t>
+          <t>SP: Av. Brig. Faria Lima, 3311, 3o andar, (11) 3288-6060 | RJ: Av. Rio Branco, 151, 5o andar, (21) 3553-1707</t>
         </is>
       </c>
       <c r="K86" s="4" t="inlineStr">
         <is>
-          <t>Atuam desde 2012 so em previdenciario, com CONSULTA ONLINE PARA TODO O BRASIL. BPC/LOAS, incapacidade, pensao por morte e revisoes - demandas do JEF de Ji-Parana.</t>
+          <t>Tem pagina CAREERS. Area declarada de Strategic Litigation and Arbitration.</t>
         </is>
       </c>
       <c r="L86" s="4" t="inlineStr">
@@ -5534,17 +5534,17 @@
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>SA Law Advogados</t>
+          <t>Select Saúde (Select Operadora)</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>São Paulo</t>
+          <t>Goiânia</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="E87" s="7" t="inlineStr">
@@ -5554,28 +5554,28 @@
       </c>
       <c r="F87" s="6" t="inlineStr">
         <is>
-          <t>+55 (11) 3288-6060</t>
+          <t>0800 224 2808</t>
         </is>
       </c>
       <c r="G87" s="4" t="inlineStr">
         <is>
-          <t>Correspondencia e candidatura (pagina Careers)</t>
+          <t>Contencioso de saude suplementar</t>
         </is>
       </c>
       <c r="H87" s="4" t="inlineStr"/>
       <c r="I87" s="4" t="inlineStr">
         <is>
-          <t>https://salaw.com.br/</t>
+          <t>https://selectoperadora.com.br/</t>
         </is>
       </c>
       <c r="J87" s="4" t="inlineStr">
         <is>
-          <t>SP: Av. Brig. Faria Lima, 3311, 3o andar, (11) 3288-6060 | RJ: Av. Rio Branco, 151, 5o andar, (21) 3553-1707</t>
+          <t>St. Oeste, Goiania-GO</t>
         </is>
       </c>
       <c r="K87" s="4" t="inlineStr">
         <is>
-          <t>Tem pagina CAREERS. Area declarada de Strategic Litigation and Arbitration.</t>
+          <t>TEM PAGINA "SEJA UM CREDENCIADO" E "SEJA NOSSO PARCEIRO" - canais formais de entrada. Opera em Porto Velho e Ji-Parana.</t>
         </is>
       </c>
       <c r="L87" s="4" t="inlineStr">
@@ -5592,17 +5592,17 @@
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>Select Saúde (Select Operadora)</t>
+          <t>Zveiter Advogados</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>Goiânia</t>
+          <t>Rio de Janeiro</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="E88" s="7" t="inlineStr">
@@ -5612,28 +5612,28 @@
       </c>
       <c r="F88" s="6" t="inlineStr">
         <is>
-          <t>0800 224 2808</t>
+          <t>55 (21) 3380-1155</t>
         </is>
       </c>
       <c r="G88" s="4" t="inlineStr">
         <is>
-          <t>Contencioso de saude suplementar</t>
+          <t>Correspondencia para as carteiras de massa</t>
         </is>
       </c>
       <c r="H88" s="4" t="inlineStr"/>
       <c r="I88" s="4" t="inlineStr">
         <is>
-          <t>https://selectoperadora.com.br/</t>
+          <t>https://zveiter.com.br/</t>
         </is>
       </c>
       <c r="J88" s="4" t="inlineStr">
         <is>
-          <t>St. Oeste, Goiania-GO</t>
+          <t>Av. Presidente Antonio Carlos, 51, 19o e 20o andares, Centro, Rio de Janeiro/RJ | Fundado em 1957</t>
         </is>
       </c>
       <c r="K88" s="4" t="inlineStr">
         <is>
-          <t>TEM PAGINA "SEJA UM CREDENCIADO" E "SEJA NOSSO PARCEIRO" - canais formais de entrada. Opera em Porto Velho e Ji-Parana.</t>
+          <t>67 anos. Atua em contencioso de massa, saude suplementar, recuperacao judicial e falencias. Conduz as RJs do Grupo Petropolis e Grupo Americanas - carteiras com credores no pais inteiro.</t>
         </is>
       </c>
       <c r="L88" s="4" t="inlineStr">
@@ -5650,48 +5650,48 @@
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>Zveiter Advogados</t>
+          <t>ABL Advogados (Aith, Badari e Luchin)</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>Rio de Janeiro</t>
+          <t>Santo André</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t>RJ</t>
-        </is>
-      </c>
-      <c r="E89" s="7" t="inlineStr">
-        <is>
-          <t>TELEFONE</t>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E89" s="10" t="inlineStr">
+        <is>
+          <t>FORMULARIO</t>
         </is>
       </c>
       <c r="F89" s="6" t="inlineStr">
         <is>
-          <t>55 (21) 3380-1155</t>
+          <t>https://abladvogados.com/</t>
         </is>
       </c>
       <c r="G89" s="4" t="inlineStr">
         <is>
-          <t>Correspondencia para as carteiras de massa</t>
+          <t>Parceria previdenciaria - pagina PARA ADVOGADOS</t>
         </is>
       </c>
       <c r="H89" s="4" t="inlineStr"/>
       <c r="I89" s="4" t="inlineStr">
         <is>
-          <t>https://zveiter.com.br/</t>
+          <t>https://abladvogados.com/</t>
         </is>
       </c>
       <c r="J89" s="4" t="inlineStr">
         <is>
-          <t>Av. Presidente Antonio Carlos, 51, 19o e 20o andares, Centro, Rio de Janeiro/RJ | Fundado em 1957</t>
+          <t>Matriz Santo Andre/SP (11) 4509-4697 | filiais: Piracaia, Extrema/MG, Rio Claro 0800 707 4697, Mogi Mirim, Santos, Atibaia, Assis, Estiva Gerbi</t>
         </is>
       </c>
       <c r="K89" s="4" t="inlineStr">
         <is>
-          <t>67 anos. Atua em contencioso de massa, saude suplementar, recuperacao judicial e falencias. Conduz as RJs do Grupo Petropolis e Grupo Americanas - carteiras com credores no pais inteiro.</t>
+          <t>TEM MENU "PARA ADVOGADOS" E "TRABALHE CONOSCO" - canal especifico para parceria entre advogados. +90 profissionais so em previdenciario. Todas as filiais no Sudeste - Norte descoberto.</t>
         </is>
       </c>
       <c r="L89" s="4" t="inlineStr">
@@ -5708,17 +5708,17 @@
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>ABL Advogados (Aith, Badari e Luchin)</t>
+          <t>Brasdiesel (Concessionária Scania)</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>Santo André</t>
+          <t>Não informado</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>BR</t>
         </is>
       </c>
       <c r="E90" s="10" t="inlineStr">
@@ -5728,28 +5728,28 @@
       </c>
       <c r="F90" s="6" t="inlineStr">
         <is>
-          <t>https://abladvogados.com/</t>
+          <t>https://www.brasdiesel.com.br/</t>
         </is>
       </c>
       <c r="G90" s="4" t="inlineStr">
         <is>
-          <t>Parceria previdenciaria - pagina PARA ADVOGADOS</t>
+          <t>Assessoria em consumidor e contratos</t>
         </is>
       </c>
       <c r="H90" s="4" t="inlineStr"/>
       <c r="I90" s="4" t="inlineStr">
         <is>
-          <t>https://abladvogados.com/</t>
+          <t>https://www.brasdiesel.com.br/</t>
         </is>
       </c>
       <c r="J90" s="4" t="inlineStr">
         <is>
-          <t>Matriz Santo Andre/SP (11) 4509-4697 | filiais: Piracaia, Extrema/MG, Rio Claro 0800 707 4697, Mogi Mirim, Santos, Atibaia, Assis, Estiva Gerbi</t>
+          <t>Paginas: Fale Conosco, TRABALHE CONOSCO, Vagas Disponiveis e COMPLIANCE BRASDIESEL</t>
         </is>
       </c>
       <c r="K90" s="4" t="inlineStr">
         <is>
-          <t>TEM MENU "PARA ADVOGADOS" E "TRABALHE CONOSCO" - canal especifico para parceria entre advogados. +90 profissionais so em previdenciario. Todas as filiais no Sudeste - Norte descoberto.</t>
+          <t>ATENCAO: este dominio e da concessionaria Scania, pode nao ser a TRR BrasDiesel de Ji-Parana do ranking Econodata - confirmar antes de abordar. Tem canal de compliance e vagas.</t>
         </is>
       </c>
       <c r="L90" s="4" t="inlineStr">
@@ -5766,17 +5766,17 @@
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>Brasdiesel (Concessionária Scania)</t>
+          <t>Energisa (grupo)</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>Não informado</t>
+          <t>Cataguases</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>MG</t>
         </is>
       </c>
       <c r="E91" s="10" t="inlineStr">
@@ -5786,28 +5786,28 @@
       </c>
       <c r="F91" s="6" t="inlineStr">
         <is>
-          <t>https://www.brasdiesel.com.br/</t>
+          <t>https://www.energisa.com.br/</t>
         </is>
       </c>
       <c r="G91" s="4" t="inlineStr">
         <is>
-          <t>Assessoria em consumidor e contratos</t>
+          <t>Defesa em acoes consumeristas nas comarcas de RO</t>
         </is>
       </c>
       <c r="H91" s="4" t="inlineStr"/>
       <c r="I91" s="4" t="inlineStr">
         <is>
-          <t>https://www.brasdiesel.com.br/</t>
+          <t>https://www.energisa.com.br/</t>
         </is>
       </c>
       <c r="J91" s="4" t="inlineStr">
         <is>
-          <t>Paginas: Fale Conosco, TRABALHE CONOSCO, Vagas Disponiveis e COMPLIANCE BRASDIESEL</t>
+          <t>Site institucional lista atuacao em RONDONIA entre os estados atendidos, com acoes em Porto Velho e JI-PARANA</t>
         </is>
       </c>
       <c r="K91" s="4" t="inlineStr">
         <is>
-          <t>ATENCAO: este dominio e da concessionaria Scania, pode nao ser a TRR BrasDiesel de Ji-Parana do ranking Econodata - confirmar antes de abordar. Tem canal de compliance e vagas.</t>
+          <t>Concessionaria de energia e um dos setores mais acionados por consumidores segundo o CNJ. Atuacao confirmada em Ji-Parana no proprio site.</t>
         </is>
       </c>
       <c r="L91" s="4" t="inlineStr">
@@ -5824,17 +5824,17 @@
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>Energisa (grupo)</t>
+          <t>JBS</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>Cataguases</t>
+          <t>São Paulo</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
         <is>
-          <t>MG</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="E92" s="10" t="inlineStr">
@@ -5844,28 +5844,28 @@
       </c>
       <c r="F92" s="6" t="inlineStr">
         <is>
-          <t>https://www.energisa.com.br/</t>
+          <t>https://www.jbs.com.br/</t>
         </is>
       </c>
       <c r="G92" s="4" t="inlineStr">
         <is>
-          <t>Defesa em acoes consumeristas nas comarcas de RO</t>
+          <t>Assessoria trabalhista e doencas ocupacionais</t>
         </is>
       </c>
       <c r="H92" s="4" t="inlineStr"/>
       <c r="I92" s="4" t="inlineStr">
         <is>
-          <t>https://www.energisa.com.br/</t>
+          <t>https://www.jbs.com.br/</t>
         </is>
       </c>
       <c r="J92" s="4" t="inlineStr">
         <is>
-          <t>Site institucional lista atuacao em RONDONIA entre os estados atendidos, com acoes em Porto Velho e JI-PARANA</t>
+          <t>+158 mil colaboradores no Brasil | +130 fabricas | presenca em 17 estados | pagina CARREIRAS</t>
         </is>
       </c>
       <c r="K92" s="4" t="inlineStr">
         <is>
-          <t>Concessionaria de energia e um dos setores mais acionados por consumidores segundo o CNJ. Atuacao confirmada em Ji-Parana no proprio site.</t>
+          <t>CINCO plantas em Rondonia (Vilhena, Sao Miguel do Guapore, Rolim de Moura, Ariquemes e Porto Velho). 158 mil empregados = passivo trabalhista e de doenca ocupacional em escala. Sua especialidade declarada.</t>
         </is>
       </c>
       <c r="L92" s="4" t="inlineStr">
@@ -5882,17 +5882,17 @@
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>JBS</t>
+          <t>Koetz Advocacia</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>São Paulo</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="E93" s="10" t="inlineStr">
@@ -5902,28 +5902,28 @@
       </c>
       <c r="F93" s="6" t="inlineStr">
         <is>
-          <t>https://www.jbs.com.br/</t>
+          <t>https://koetzadvocacia.com.br/</t>
         </is>
       </c>
       <c r="G93" s="4" t="inlineStr">
         <is>
-          <t>Assessoria trabalhista e doencas ocupacionais</t>
+          <t>Correspondencia previdenciaria em RO</t>
         </is>
       </c>
       <c r="H93" s="4" t="inlineStr"/>
       <c r="I93" s="4" t="inlineStr">
         <is>
-          <t>https://www.jbs.com.br/</t>
+          <t>https://koetzadvocacia.com.br/</t>
         </is>
       </c>
       <c r="J93" s="4" t="inlineStr">
         <is>
-          <t>+158 mil colaboradores no Brasil | +130 fabricas | presenca em 17 estados | pagina CARREIRAS</t>
+          <t>Contato pelo site | Eduardo Koetz (fundador), Murilo Mella (CEO)</t>
         </is>
       </c>
       <c r="K93" s="4" t="inlineStr">
         <is>
-          <t>CINCO plantas em Rondonia (Vilhena, Sao Miguel do Guapore, Rolim de Moura, Ariquemes e Porto Velho). 158 mil empregados = passivo trabalhista e de doenca ocupacional em escala. Sua especialidade declarada.</t>
+          <t>"Atendemos ONLINE qualquer pessoa em QUALQUER LUGAR DO MUNDO". Aposentadoria complexa e internacional. Operacao 100% digital precisa de presenca fisica para pericia e audiencia no JEF.</t>
         </is>
       </c>
       <c r="L93" s="4" t="inlineStr">
@@ -5940,17 +5940,17 @@
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>Koetz Advocacia</t>
+          <t>Parish &amp; Zenandro Advogados</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>Salvador</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="E94" s="10" t="inlineStr">
@@ -5960,28 +5960,28 @@
       </c>
       <c r="F94" s="6" t="inlineStr">
         <is>
-          <t>https://koetzadvocacia.com.br/</t>
+          <t>https://pz.adv.br/</t>
         </is>
       </c>
       <c r="G94" s="4" t="inlineStr">
         <is>
-          <t>Correspondencia previdenciaria em RO</t>
+          <t>Correspondencia previdenciaria e do servidor</t>
         </is>
       </c>
       <c r="H94" s="4" t="inlineStr"/>
       <c r="I94" s="4" t="inlineStr">
         <is>
-          <t>https://koetzadvocacia.com.br/</t>
+          <t>https://pz.adv.br/</t>
         </is>
       </c>
       <c r="J94" s="4" t="inlineStr">
         <is>
-          <t>Contato pelo site | Eduardo Koetz (fundador), Murilo Mella (CEO)</t>
+          <t>Matriz Salvador: Rua Frederico Simoes, 153, 13o andar, Caminho das Arvores | Unidades: Serrinha, Monte Gordo/Camacari, Retirolandia, Sao Goncalo dos Campos, Santaluz, Camacari, Feira de Santana</t>
         </is>
       </c>
       <c r="K94" s="4" t="inlineStr">
         <is>
-          <t>"Atendemos ONLINE qualquer pessoa em QUALQUER LUGAR DO MUNDO". Aposentadoria complexa e internacional. Operacao 100% digital precisa de presenca fisica para pericia e audiencia no JEF.</t>
+          <t>88 PROFISSIONAIS na equipe juridica, todos concentrados na Bahia. Previdenciario, consumidor e trabalhista. Expansao para fora do estado exigiria parceiro local.</t>
         </is>
       </c>
       <c r="L94" s="4" t="inlineStr">
@@ -5998,17 +5998,17 @@
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>Parish &amp; Zenandro Advogados</t>
+          <t>Vitorino &amp; Murta Advogados</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>Salvador</t>
+          <t>Manaus</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>AM</t>
         </is>
       </c>
       <c r="E95" s="10" t="inlineStr">
@@ -6018,28 +6018,28 @@
       </c>
       <c r="F95" s="6" t="inlineStr">
         <is>
-          <t>https://pz.adv.br/</t>
+          <t>https://vitorinoemurta.com.br/</t>
         </is>
       </c>
       <c r="G95" s="4" t="inlineStr">
         <is>
-          <t>Correspondencia previdenciaria e do servidor</t>
+          <t>Correspondencia bancaria em RO</t>
         </is>
       </c>
       <c r="H95" s="4" t="inlineStr"/>
       <c r="I95" s="4" t="inlineStr">
         <is>
-          <t>https://pz.adv.br/</t>
+          <t>https://vitorinoemurta.com.br/escritorio-em-manaus/</t>
         </is>
       </c>
       <c r="J95" s="4" t="inlineStr">
         <is>
-          <t>Matriz Salvador: Rua Frederico Simoes, 153, 13o andar, Caminho das Arvores | Unidades: Serrinha, Monte Gordo/Camacari, Retirolandia, Sao Goncalo dos Campos, Santaluz, Camacari, Feira de Santana</t>
+          <t>Contato por WhatsApp pelo site | Escritorios em Manaus, Sao Paulo, Brasilia, Florianopolis e Vila Velha</t>
         </is>
       </c>
       <c r="K95" s="4" t="inlineStr">
         <is>
-          <t>88 PROFISSIONAIS na equipe juridica, todos concentrados na Bahia. Previdenciario, consumidor e trabalhista. Expansao para fora do estado exigiria parceiro local.</t>
+          <t>Maior banca de direito bancario do Norte. Atua em gestao de passivos bancarios e tributarios e execucao fiscal. Cinco pracas, nenhuma em RO.</t>
         </is>
       </c>
       <c r="L95" s="4" t="inlineStr">
@@ -6056,48 +6056,48 @@
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>Vitorino &amp; Murta Advogados</t>
+          <t>Jurídico Certo</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>Manaus</t>
+          <t>Não informado</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
         <is>
-          <t>AM</t>
-        </is>
-      </c>
-      <c r="E96" s="10" t="inlineStr">
-        <is>
-          <t>FORMULARIO</t>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="E96" s="8" t="inlineStr">
+        <is>
+          <t>PORTAL</t>
         </is>
       </c>
       <c r="F96" s="6" t="inlineStr">
         <is>
-          <t>https://vitorinoemurta.com.br/</t>
+          <t>https://www.juridicocerto.com/cadastro-advogados-correspondentes-juridicos</t>
         </is>
       </c>
       <c r="G96" s="4" t="inlineStr">
         <is>
-          <t>Correspondencia bancaria em RO</t>
+          <t>Cadastro como correspondente</t>
         </is>
       </c>
       <c r="H96" s="4" t="inlineStr"/>
       <c r="I96" s="4" t="inlineStr">
         <is>
-          <t>https://vitorinoemurta.com.br/escritorio-em-manaus/</t>
+          <t>https://www.juridicocerto.com/cadastro-advogados-correspondentes-juridicos</t>
         </is>
       </c>
       <c r="J96" s="4" t="inlineStr">
         <is>
-          <t>Contato por WhatsApp pelo site | Escritorios em Manaus, Sao Paulo, Brasilia, Florianopolis e Vila Velha</t>
+          <t>Plano Premium a partir de R$ 49/mes (anual). Cadastro inicial pede nome, e-mail profissional e senha</t>
         </is>
       </c>
       <c r="K96" s="4" t="inlineStr">
         <is>
-          <t>Maior banca de direito bancario do Norte. Atua em gestao de passivos bancarios e tributarios e execucao fiscal. Cinco pracas, nenhuma em RO.</t>
+          <t>Tem o "Juridico Pag", que garante previsibilidade de recebimento. Algoritmo encaminha demandas proximas da sua localizacao. App avisa nova demanda.</t>
         </is>
       </c>
       <c r="L96" s="4" t="inlineStr">
@@ -6107,55 +6107,55 @@
       </c>
     </row>
     <row r="97" ht="62" customHeight="1">
-      <c r="A97" s="10" t="inlineStr">
-        <is>
-          <t>4. BANCA NACIONAL — ofereça correspondência em RO</t>
+      <c r="A97" s="11" t="inlineStr">
+        <is>
+          <t>5. BPO / TERCEIRIZAÇÃO — ofereça seu serviço</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>Jurídico Certo</t>
+          <t>Juridigital (Drive Digital)</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>Não informado</t>
+          <t>Belo Horizonte</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
         <is>
-          <t>BR</t>
-        </is>
-      </c>
-      <c r="E97" s="8" t="inlineStr">
-        <is>
-          <t>PORTAL</t>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E97" s="5" t="inlineStr">
+        <is>
+          <t>E-MAIL</t>
         </is>
       </c>
       <c r="F97" s="6" t="inlineStr">
         <is>
-          <t>https://www.juridicocerto.com/cadastro-advogados-correspondentes-juridicos</t>
+          <t>relacionamento@juridigital.com.br</t>
         </is>
       </c>
       <c r="G97" s="4" t="inlineStr">
         <is>
-          <t>Cadastro como correspondente</t>
+          <t>Rede de BPO juridico e correspondencia</t>
         </is>
       </c>
       <c r="H97" s="4" t="inlineStr"/>
       <c r="I97" s="4" t="inlineStr">
         <is>
-          <t>https://www.juridicocerto.com/cadastro-advogados-correspondentes-juridicos</t>
+          <t>https://www.juridigital.com.br/bpo-juridico/</t>
         </is>
       </c>
       <c r="J97" s="4" t="inlineStr">
         <is>
-          <t>Plano Premium a partir de R$ 49/mes (anual). Cadastro inicial pede nome, e-mail profissional e senha</t>
+          <t>WhatsApp (31) 99362-8269 | Belo Horizonte/MG | CNPJ 28.407.867/0001-85</t>
         </is>
       </c>
       <c r="K97" s="4" t="inlineStr">
         <is>
-          <t>Tem o "Juridico Pag", que garante previsibilidade de recebimento. Algoritmo encaminha demandas proximas da sua localizacao. App avisa nova demanda.</t>
+          <t>Produzem conteudo sobre BPO juridico E sobre contratacao de correspondente juridico - conhecem e intermediam os dois mercados. Base de escritorios clientes.</t>
         </is>
       </c>
       <c r="L97" s="4" t="inlineStr">
@@ -6172,48 +6172,48 @@
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>Juridigital (Drive Digital)</t>
+          <t>CSilva Sociedade de Advogados (BPO.CS)</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>Belo Horizonte</t>
+          <t>Não informado</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>MG</t>
-        </is>
-      </c>
-      <c r="E98" s="5" t="inlineStr">
-        <is>
-          <t>E-MAIL</t>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="E98" s="10" t="inlineStr">
+        <is>
+          <t>FORMULARIO</t>
         </is>
       </c>
       <c r="F98" s="6" t="inlineStr">
         <is>
-          <t>relacionamento@juridigital.com.br</t>
+          <t>https://csilvaadv.com.br/terceirizacao-de-servicos-juridicos/</t>
         </is>
       </c>
       <c r="G98" s="4" t="inlineStr">
         <is>
-          <t>Rede de BPO juridico e correspondencia</t>
+          <t>Prestacao de servico para a operacao de BPO</t>
         </is>
       </c>
       <c r="H98" s="4" t="inlineStr"/>
       <c r="I98" s="4" t="inlineStr">
         <is>
-          <t>https://www.juridigital.com.br/bpo-juridico/</t>
+          <t>https://csilvaadv.com.br/terceirizacao-de-servicos-juridicos/</t>
         </is>
       </c>
       <c r="J98" s="4" t="inlineStr">
         <is>
-          <t>WhatsApp (31) 99362-8269 | Belo Horizonte/MG | CNPJ 28.407.867/0001-85</t>
+          <t>Contato via WhatsApp pelo site</t>
         </is>
       </c>
       <c r="K98" s="4" t="inlineStr">
         <is>
-          <t>Produzem conteudo sobre BPO juridico E sobre contratacao de correspondente juridico - conhecem e intermediam os dois mercados. Base de escritorios clientes.</t>
+          <t>Escritorio especializado em BPO Juridico para empresas de todos os portes.</t>
         </is>
       </c>
       <c r="L98" s="4" t="inlineStr">
@@ -6230,17 +6230,17 @@
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>CSilva Sociedade de Advogados (BPO.CS)</t>
+          <t>Carbonera &amp; Tomazini Advogados</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>Não informado</t>
+          <t>Gravataí</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="E99" s="10" t="inlineStr">
@@ -6250,28 +6250,28 @@
       </c>
       <c r="F99" s="6" t="inlineStr">
         <is>
-          <t>https://csilvaadv.com.br/terceirizacao-de-servicos-juridicos/</t>
+          <t>https://www.carboneraetomazini.com.br/</t>
         </is>
       </c>
       <c r="G99" s="4" t="inlineStr">
         <is>
-          <t>Prestacao de servico para a operacao de BPO</t>
+          <t>PARCERIA EM DIREITO PREVIDENCIARIO (pagina propria)</t>
         </is>
       </c>
       <c r="H99" s="4" t="inlineStr"/>
       <c r="I99" s="4" t="inlineStr">
         <is>
-          <t>https://csilvaadv.com.br/terceirizacao-de-servicos-juridicos/</t>
+          <t>https://www.carboneraetomazini.com.br/</t>
         </is>
       </c>
       <c r="J99" s="4" t="inlineStr">
         <is>
-          <t>Contato via WhatsApp pelo site</t>
+          <t>Matriz Gravatai/RS (51) 3933-6733 | Filiais: Joinville (47) 3028-8555 e (47) 3017-5941, Rio Grande (53) 3035-3615, Fortaleza (85) 3032-4886 e (85) 3122-3878 | Escritorio Digital: (51) 3424-3615, (51) 99726-5382, (51) 99667-0941, (51) 99881-3738, (85) 98823-8227, (47) 98924-3140, (53) 99130-4900 | CNPJ 20.920.282/0001-52</t>
         </is>
       </c>
       <c r="K99" s="4" t="inlineStr">
         <is>
-          <t>Escritorio especializado em BPO Juridico para empresas de todos os portes.</t>
+          <t>MELHOR ACHADO DA RODADA: o menu do site tem item proprio "PARCERIA EM DIREITO PREVIDENCIARIO" e tambem "Trabalhe Conosco". Atendem todo o Brasil pelo Escritorio Digital. OAB/RS 5.067 e OAB/SC 4.029. Previdenciario e sua area principal.</t>
         </is>
       </c>
       <c r="L99" s="4" t="inlineStr">
@@ -6288,17 +6288,17 @@
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>Carbonera &amp; Tomazini Advogados</t>
+          <t>Ehts Consulting</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>Gravataí</t>
+          <t>Não informado</t>
         </is>
       </c>
       <c r="D100" s="4" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>BR</t>
         </is>
       </c>
       <c r="E100" s="10" t="inlineStr">
@@ -6308,28 +6308,28 @@
       </c>
       <c r="F100" s="6" t="inlineStr">
         <is>
-          <t>https://www.carboneraetomazini.com.br/</t>
+          <t>https://ehts.com.br/quem-somos/</t>
         </is>
       </c>
       <c r="G100" s="4" t="inlineStr">
         <is>
-          <t>PARCERIA EM DIREITO PREVIDENCIARIO (pagina propria)</t>
+          <t>Prestacao de servico em legal operations</t>
         </is>
       </c>
       <c r="H100" s="4" t="inlineStr"/>
       <c r="I100" s="4" t="inlineStr">
         <is>
-          <t>https://www.carboneraetomazini.com.br/</t>
+          <t>https://ehts.com.br/quem-somos/</t>
         </is>
       </c>
       <c r="J100" s="4" t="inlineStr">
         <is>
-          <t>Matriz Gravatai/RS (51) 3933-6733 | Filiais: Joinville (47) 3028-8555 e (47) 3017-5941, Rio Grande (53) 3035-3615, Fortaleza (85) 3032-4886 e (85) 3122-3878 | Escritorio Digital: (51) 3424-3615, (51) 99726-5382, (51) 99667-0941, (51) 99881-3738, (85) 98823-8227, (47) 98924-3140, (53) 99130-4900 | CNPJ 20.920.282/0001-52</t>
+          <t>Contato pelo site e WhatsApp</t>
         </is>
       </c>
       <c r="K100" s="4" t="inlineStr">
         <is>
-          <t>MELHOR ACHADO DA RODADA: o menu do site tem item proprio "PARCERIA EM DIREITO PREVIDENCIARIO" e tambem "Trabalhe Conosco". Atendem todo o Brasil pelo Escritorio Digital. OAB/RS 5.067 e OAB/SC 4.029. Previdenciario e sua area principal.</t>
+          <t>Top 10 LegalTech do Brasil (Ranking 100 Open Startups). Clientes: Petrobras, Porto Seguro, Eurofarma, Renner, Centauro, Nike, Airbnb. Legal Operations e Analytics Juridico - carteiras enormes que precisam de maos.</t>
         </is>
       </c>
       <c r="L100" s="4" t="inlineStr">
@@ -6346,17 +6346,17 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>Ehts Consulting</t>
+          <t>Intelligenti Stefanini - Locação de Headcounts</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>Não informado</t>
+          <t>São Paulo</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="E101" s="10" t="inlineStr">
@@ -6366,28 +6366,28 @@
       </c>
       <c r="F101" s="6" t="inlineStr">
         <is>
-          <t>https://ehts.com.br/quem-somos/</t>
+          <t>https://www.intelligenti.com.br/solucoes/bpo-juridico</t>
         </is>
       </c>
       <c r="G101" s="4" t="inlineStr">
         <is>
-          <t>Prestacao de servico em legal operations</t>
+          <t>Alocacao como profissional juridico (headcount)</t>
         </is>
       </c>
       <c r="H101" s="4" t="inlineStr"/>
       <c r="I101" s="4" t="inlineStr">
         <is>
-          <t>https://ehts.com.br/quem-somos/</t>
+          <t>https://www.intelligenti.com.br/solucoes/bpo-juridico</t>
         </is>
       </c>
       <c r="J101" s="4" t="inlineStr">
         <is>
-          <t>Contato pelo site e WhatsApp</t>
+          <t>Av. Eusebio Matoso, 1375, Sao Paulo/SP | Grupo Stefanini</t>
         </is>
       </c>
       <c r="K101" s="4" t="inlineStr">
         <is>
-          <t>Top 10 LegalTech do Brasil (Ranking 100 Open Startups). Clientes: Petrobras, Porto Seguro, Eurofarma, Renner, Centauro, Nike, Airbnb. Legal Operations e Analytics Juridico - carteiras enormes que precisam de maos.</t>
+          <t>MODELO IDEAL PARA RENDA EXTRA: tem servico declarado de "LOCACAO DE HEADCOUNTS - acesso rapido e flexivel a profissionais qualificados do setor juridico". Eles alocam advogados sob demanda. Ofereca-se como headcount disponivel.</t>
         </is>
       </c>
       <c r="L101" s="4" t="inlineStr">
@@ -6404,17 +6404,17 @@
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>Intelligenti Stefanini - Locação de Headcounts</t>
+          <t>Lima &amp; Pegolo Advogados (LPADV)</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>São Paulo</t>
+          <t>Não informado</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>BR</t>
         </is>
       </c>
       <c r="E102" s="10" t="inlineStr">
@@ -6424,28 +6424,28 @@
       </c>
       <c r="F102" s="6" t="inlineStr">
         <is>
-          <t>https://www.intelligenti.com.br/solucoes/bpo-juridico</t>
+          <t>https://limaepegolo.com.br/seja-um-parceiro/</t>
         </is>
       </c>
       <c r="G102" s="4" t="inlineStr">
         <is>
-          <t>Alocacao como profissional juridico (headcount)</t>
+          <t>Parceria com plataforma e teses prontas</t>
         </is>
       </c>
       <c r="H102" s="4" t="inlineStr"/>
       <c r="I102" s="4" t="inlineStr">
         <is>
-          <t>https://www.intelligenti.com.br/solucoes/bpo-juridico</t>
+          <t>https://limaepegolo.com.br/seja-um-parceiro/</t>
         </is>
       </c>
       <c r="J102" s="4" t="inlineStr">
         <is>
-          <t>Av. Eusebio Matoso, 1375, Sao Paulo/SP | Grupo Stefanini</t>
+          <t>Formulario na pagina "Seja um Parceiro"</t>
         </is>
       </c>
       <c r="K102" s="4" t="inlineStr">
         <is>
-          <t>MODELO IDEAL PARA RENDA EXTRA: tem servico declarado de "LOCACAO DE HEADCOUNTS - acesso rapido e flexivel a profissionais qualificados do setor juridico". Eles alocam advogados sob demanda. Ofereca-se como headcount disponivel.</t>
+          <t>MODELO INTERESSANTE: voce capta o cliente, eles assumem o trabalho tecnico. Texto do site: "uma vez validada a nova contratacao, TODO O TRABALHO SERA NOSSO". Da acesso a area restrita com teses do escritorio. Renda sem carga processual.</t>
         </is>
       </c>
       <c r="L102" s="4" t="inlineStr">
@@ -6462,7 +6462,7 @@
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>Lima &amp; Pegolo Advogados (LPADV)</t>
+          <t>Souza Cruz Advogados - BPO Jurídico</t>
         </is>
       </c>
       <c r="C103" s="4" t="inlineStr">
@@ -6482,28 +6482,28 @@
       </c>
       <c r="F103" s="6" t="inlineStr">
         <is>
-          <t>https://limaepegolo.com.br/seja-um-parceiro/</t>
+          <t>https://souzacruz.adv.br/bpo-juridico/</t>
         </is>
       </c>
       <c r="G103" s="4" t="inlineStr">
         <is>
-          <t>Parceria com plataforma e teses prontas</t>
+          <t>Prestacao de servico para a operacao de BPO trabalhista</t>
         </is>
       </c>
       <c r="H103" s="4" t="inlineStr"/>
       <c r="I103" s="4" t="inlineStr">
         <is>
-          <t>https://limaepegolo.com.br/seja-um-parceiro/</t>
+          <t>https://souzacruz.adv.br/bpo-juridico/</t>
         </is>
       </c>
       <c r="J103" s="4" t="inlineStr">
         <is>
-          <t>Formulario na pagina "Seja um Parceiro"</t>
+          <t>Contato pelo site com a Dra. Mariana Cruz</t>
         </is>
       </c>
       <c r="K103" s="4" t="inlineStr">
         <is>
-          <t>MODELO INTERESSANTE: voce capta o cliente, eles assumem o trabalho tecnico. Texto do site: "uma vez validada a nova contratacao, TODO O TRABALHO SERA NOSSO". Da acesso a area restrita com teses do escritorio. Renda sem carga processual.</t>
+          <t>BPO trabalhista que atende escritorios e departamentos juridicos: controladoria, gestao de prazos, acompanhamento processual, elaboracao de pecas e sustentacoes. Eles COMPRAM o servico que voce vende.</t>
         </is>
       </c>
       <c r="L103" s="4" t="inlineStr">
@@ -6513,60 +6513,64 @@
       </c>
     </row>
     <row r="104" ht="62" customHeight="1">
-      <c r="A104" s="11" t="inlineStr">
-        <is>
-          <t>5. BPO / TERCEIRIZAÇÃO — ofereça seu serviço</t>
+      <c r="A104" s="12" t="inlineStr">
+        <is>
+          <t>6. VAGA ABERTA — candidate-se</t>
         </is>
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>Souza Cruz Advogados - BPO Jurídico</t>
+          <t>Carlos Miro Advogados</t>
         </is>
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>Não informado</t>
+          <t>Uberlândia</t>
         </is>
       </c>
       <c r="D104" s="4" t="inlineStr">
         <is>
-          <t>BR</t>
-        </is>
-      </c>
-      <c r="E104" s="10" t="inlineStr">
-        <is>
-          <t>FORMULARIO</t>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E104" s="5" t="inlineStr">
+        <is>
+          <t>E-MAIL</t>
         </is>
       </c>
       <c r="F104" s="6" t="inlineStr">
         <is>
-          <t>https://souzacruz.adv.br/bpo-juridico/</t>
+          <t>yasminsantos@carlosmiro.adv.br</t>
         </is>
       </c>
       <c r="G104" s="4" t="inlineStr">
         <is>
-          <t>Prestacao de servico para a operacao de BPO trabalhista</t>
-        </is>
-      </c>
-      <c r="H104" s="4" t="inlineStr"/>
+          <t>Advogado Contencioso Massificado</t>
+        </is>
+      </c>
+      <c r="H104" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
       <c r="I104" s="4" t="inlineStr">
         <is>
-          <t>https://souzacruz.adv.br/bpo-juridico/</t>
+          <t>https://to.indeed.com/aanzcqdqkn8x</t>
         </is>
       </c>
       <c r="J104" s="4" t="inlineStr">
         <is>
-          <t>Contato pelo site com a Dra. Mariana Cruz</t>
+          <t>"Interessados na oportunidade podem se cadastrar por aqui ou enviar o curriculo para o e-mail yasminsantos@carlosmiro.adv.br"</t>
         </is>
       </c>
       <c r="K104" s="4" t="inlineStr">
         <is>
-          <t>BPO trabalhista que atende escritorios e departamentos juridicos: controladoria, gestao de prazos, acompanhamento processual, elaboracao de pecas e sustentacoes. Eles COMPRAM o servico que voce vende.</t>
+          <t>50 anos de mercado, bancario e empresarial. O anuncio diz que ja opera com CORRESPONDENTES em diversas localidades do pais - vale ofertar RO na mesma mensagem.</t>
         </is>
       </c>
       <c r="L104" s="4" t="inlineStr">
         <is>
-          <t>Site institucional (extracao Tavily)</t>
+          <t>Descricao completa da vaga no Indeed (get_job_details)</t>
         </is>
       </c>
     </row>
@@ -6578,17 +6582,17 @@
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>Carlos Miro Advogados</t>
+          <t>Carneiro &amp; Ramalho Consultoria (p/ NEST Construções)</t>
         </is>
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>Uberlândia</t>
+          <t>Jaboatão dos Guararapes</t>
         </is>
       </c>
       <c r="D105" s="4" t="inlineStr">
         <is>
-          <t>MG</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
@@ -6598,32 +6602,32 @@
       </c>
       <c r="F105" s="6" t="inlineStr">
         <is>
-          <t>yasminsantos@carlosmiro.adv.br</t>
+          <t>consultoraselecaopb@gmail.com</t>
         </is>
       </c>
       <c r="G105" s="4" t="inlineStr">
         <is>
-          <t>Advogado Contencioso Massificado</t>
+          <t>Advogado(a) Associado(a)</t>
         </is>
       </c>
       <c r="H105" s="4" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="I105" s="4" t="inlineStr">
         <is>
-          <t>https://to.indeed.com/aanzcqdqkn8x</t>
+          <t>https://to.indeed.com/aagvvpqgq4h9</t>
         </is>
       </c>
       <c r="J105" s="4" t="inlineStr">
         <is>
-          <t>"Interessados na oportunidade podem se cadastrar por aqui ou enviar o curriculo para o e-mail yasminsantos@carlosmiro.adv.br"</t>
+          <t>"Enviar o curriculo para o e-mail: consultoraselecaopb@gmail.com"</t>
         </is>
       </c>
       <c r="K105" s="4" t="inlineStr">
         <is>
-          <t>50 anos de mercado, bancario e empresarial. O anuncio diz que ja opera com CORRESPONDENTES em diversas localidades do pais - vale ofertar RO na mesma mensagem.</t>
+          <t>Civel, execucao e cobranca, audiencias.</t>
         </is>
       </c>
       <c r="L105" s="4" t="inlineStr">
@@ -6640,17 +6644,17 @@
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t>Carneiro &amp; Ramalho Consultoria (p/ NEST Construções)</t>
+          <t>Décio Freire Advogados</t>
         </is>
       </c>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>Jaboatão dos Guararapes</t>
+          <t>Teresina</t>
         </is>
       </c>
       <c r="D106" s="4" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="E106" s="5" t="inlineStr">
@@ -6660,32 +6664,32 @@
       </c>
       <c r="F106" s="6" t="inlineStr">
         <is>
-          <t>consultoraselecaopb@gmail.com</t>
+          <t>christianedepaula@deciofreire.com.br</t>
         </is>
       </c>
       <c r="G106" s="4" t="inlineStr">
         <is>
-          <t>Advogado(a) Associado(a)</t>
+          <t>Advogado(a) Civel PLENO - Unidade Teresina (PJ)</t>
         </is>
       </c>
       <c r="H106" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="I106" s="4" t="inlineStr">
         <is>
-          <t>https://to.indeed.com/aagvvpqgq4h9</t>
+          <t>https://to.indeed.com/aasphhw2vxx4</t>
         </is>
       </c>
       <c r="J106" s="4" t="inlineStr">
         <is>
-          <t>"Enviar o curriculo para o e-mail: consultoraselecaopb@gmail.com"</t>
+          <t>"Os(as) interessados(as) deverao encaminhar o curriculo informando a pretensao de honorarios para o e-mail christianedepaula@deciofreire.com.br"</t>
         </is>
       </c>
       <c r="K106" s="4" t="inlineStr">
         <is>
-          <t>Civel, execucao e cobranca, audiencias.</t>
+          <t>Banca nacional com escritorios em SP, RJ, BH, Brasilia e Recife. Exige informar pretensao de honorarios. Contratacao PJ.</t>
         </is>
       </c>
       <c r="L106" s="4" t="inlineStr">
@@ -6702,17 +6706,17 @@
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>Décio Freire Advogados</t>
+          <t>GWF Advogados e Associados</t>
         </is>
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>Teresina</t>
+          <t>Ribeirão Preto</t>
         </is>
       </c>
       <c r="D107" s="4" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="E107" s="5" t="inlineStr">
@@ -6722,32 +6726,32 @@
       </c>
       <c r="F107" s="6" t="inlineStr">
         <is>
-          <t>christianedepaula@deciofreire.com.br</t>
+          <t>gestao@gwfadvocacia.com.br</t>
         </is>
       </c>
       <c r="G107" s="4" t="inlineStr">
         <is>
-          <t>Advogado(a) Civel PLENO - Unidade Teresina (PJ)</t>
+          <t>Advogado(a) Senior Lider - Direito Bancario</t>
         </is>
       </c>
       <c r="H107" s="4" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="I107" s="4" t="inlineStr">
         <is>
-          <t>https://to.indeed.com/aasphhw2vxx4</t>
+          <t>https://to.indeed.com/aa6ntjfd4f72</t>
         </is>
       </c>
       <c r="J107" s="4" t="inlineStr">
         <is>
-          <t>"Os(as) interessados(as) deverao encaminhar o curriculo informando a pretensao de honorarios para o e-mail christianedepaula@deciofreire.com.br"</t>
+          <t>"Interessados podem encaminhar o curriculo para: gestao@gwfadvocacia.com.br"</t>
         </is>
       </c>
       <c r="K107" s="4" t="inlineStr">
         <is>
-          <t>Banca nacional com escritorios em SP, RJ, BH, Brasilia e Recife. Exige informar pretensao de honorarios. Contratacao PJ.</t>
+          <t>Bancario e contencioso civel. Faixa ate R$ 15.000.</t>
         </is>
       </c>
       <c r="L107" s="4" t="inlineStr">
@@ -6764,17 +6768,17 @@
       </c>
       <c r="B108" s="3" t="inlineStr">
         <is>
-          <t>GWF Advogados e Associados</t>
+          <t>Gonçalves Júnior Advocacia</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>Ribeirão Preto</t>
+          <t>Brasília</t>
         </is>
       </c>
       <c r="D108" s="4" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>DF</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">
@@ -6784,32 +6788,32 @@
       </c>
       <c r="F108" s="6" t="inlineStr">
         <is>
-          <t>gestao@gwfadvocacia.com.br</t>
+          <t>contato@goncalvesjunioradv.com</t>
         </is>
       </c>
       <c r="G108" s="4" t="inlineStr">
         <is>
-          <t>Advogado(a) Senior Lider - Direito Bancario</t>
+          <t>Advogado(a) Associado(a) - Civel/Tributario | ATUACAO INICIAL REMOTA</t>
         </is>
       </c>
       <c r="H108" s="4" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="I108" s="4" t="inlineStr">
         <is>
-          <t>https://to.indeed.com/aa6ntjfd4f72</t>
+          <t>https://to.indeed.com/aaw8gpwjhqy7</t>
         </is>
       </c>
       <c r="J108" s="4" t="inlineStr">
         <is>
-          <t>"Interessados podem encaminhar o curriculo para: gestao@gwfadvocacia.com.br"</t>
+          <t>"Os interessados deverao enviar curriculo para: contato@goncalvesjunioradv.com - Assunto: Processo Seletivo - Advogado(a) Associado(a) - Civel/Tributario"</t>
         </is>
       </c>
       <c r="K108" s="4" t="inlineStr">
         <is>
-          <t>Bancario e contencioso civel. Faixa ate R$ 15.000.</t>
+          <t>ATENCAO: o prazo do anuncio era 10/09/2026. Mas o proprio texto diz que aprovados ficam em cadastro por ate 6 meses - vale enviar assim mesmo.</t>
         </is>
       </c>
       <c r="L108" s="4" t="inlineStr">
@@ -6826,17 +6830,17 @@
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>Gonçalves Júnior Advocacia</t>
+          <t>Marcelo Tostes Advogados Associados</t>
         </is>
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>Brasília</t>
+          <t>Belo Horizonte</t>
         </is>
       </c>
       <c r="D109" s="4" t="inlineStr">
         <is>
-          <t>DF</t>
+          <t>MG</t>
         </is>
       </c>
       <c r="E109" s="5" t="inlineStr">
@@ -6846,32 +6850,32 @@
       </c>
       <c r="F109" s="6" t="inlineStr">
         <is>
-          <t>contato@goncalvesjunioradv.com</t>
+          <t>recrutamento@mtostes.com.br</t>
         </is>
       </c>
       <c r="G109" s="4" t="inlineStr">
         <is>
-          <t>Advogado(a) Associado(a) - Civel/Tributario | ATUACAO INICIAL REMOTA</t>
+          <t>Advogado Civel Junior / Pleno - Contencioso de Escala</t>
         </is>
       </c>
       <c r="H109" s="4" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="I109" s="4" t="inlineStr">
         <is>
-          <t>https://to.indeed.com/aaw8gpwjhqy7</t>
+          <t>https://to.indeed.com/aazhlrrjljqn</t>
         </is>
       </c>
       <c r="J109" s="4" t="inlineStr">
         <is>
-          <t>"Os interessados deverao enviar curriculo para: contato@goncalvesjunioradv.com - Assunto: Processo Seletivo - Advogado(a) Associado(a) - Civel/Tributario"</t>
+          <t>"Candidate-se ou envie seu curriculo para recrutamento@mtostes.com.br indicando no assunto Advogado Civel - BH"</t>
         </is>
       </c>
       <c r="K109" s="4" t="inlineStr">
         <is>
-          <t>ATENCAO: o prazo do anuncio era 10/09/2026. Mas o proprio texto diz que aprovados ficam em cadastro por ate 6 meses - vale enviar assim mesmo.</t>
+          <t>Banca nacional de contencioso de massa e recuperacao de credito. Colocar o assunto pedido.</t>
         </is>
       </c>
       <c r="L109" s="4" t="inlineStr">
@@ -6888,12 +6892,12 @@
       </c>
       <c r="B110" s="3" t="inlineStr">
         <is>
-          <t>Marcelo Tostes Advogados Associados</t>
+          <t>Reis Advogados Associados</t>
         </is>
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>Belo Horizonte</t>
+          <t>Uberlândia</t>
         </is>
       </c>
       <c r="D110" s="4" t="inlineStr">
@@ -6901,19 +6905,19 @@
           <t>MG</t>
         </is>
       </c>
-      <c r="E110" s="5" t="inlineStr">
-        <is>
-          <t>E-MAIL</t>
+      <c r="E110" s="8" t="inlineStr">
+        <is>
+          <t>PORTAL</t>
         </is>
       </c>
       <c r="F110" s="6" t="inlineStr">
         <is>
-          <t>recrutamento@mtostes.com.br</t>
+          <t>https://reisadvogados.vagas.solides.com.br/vaga/915401</t>
         </is>
       </c>
       <c r="G110" s="4" t="inlineStr">
         <is>
-          <t>Advogado Civel Junior / Pleno - Contencioso de Escala</t>
+          <t>Assistente de Controladoria Juridica (PJ)</t>
         </is>
       </c>
       <c r="H110" s="4" t="inlineStr">
@@ -6923,17 +6927,17 @@
       </c>
       <c r="I110" s="4" t="inlineStr">
         <is>
-          <t>https://to.indeed.com/aazhlrrjljqn</t>
+          <t>https://to.indeed.com/aay7xrjqdxpw</t>
         </is>
       </c>
       <c r="J110" s="4" t="inlineStr">
         <is>
-          <t>"Candidate-se ou envie seu curriculo para recrutamento@mtostes.com.br indicando no assunto Advogado Civel - BH"</t>
+          <t>"REALIZAR CANDIDATURA NO LINK: https://reisadvogados.vagas.solides.com.br/vaga/915401"</t>
         </is>
       </c>
       <c r="K110" s="4" t="inlineStr">
         <is>
-          <t>Banca nacional de contencioso de massa e recuperacao de credito. Colocar o assunto pedido.</t>
+          <t>Candidatura so pelo link proprio, nao pelo Indeed.</t>
         </is>
       </c>
       <c r="L110" s="4" t="inlineStr">
@@ -6942,68 +6946,7 @@
         </is>
       </c>
     </row>
-    <row r="111" ht="62" customHeight="1">
-      <c r="A111" s="12" t="inlineStr">
-        <is>
-          <t>6. VAGA ABERTA — candidate-se</t>
-        </is>
-      </c>
-      <c r="B111" s="3" t="inlineStr">
-        <is>
-          <t>Reis Advogados Associados</t>
-        </is>
-      </c>
-      <c r="C111" s="4" t="inlineStr">
-        <is>
-          <t>Uberlândia</t>
-        </is>
-      </c>
-      <c r="D111" s="4" t="inlineStr">
-        <is>
-          <t>MG</t>
-        </is>
-      </c>
-      <c r="E111" s="8" t="inlineStr">
-        <is>
-          <t>PORTAL</t>
-        </is>
-      </c>
-      <c r="F111" s="6" t="inlineStr">
-        <is>
-          <t>https://reisadvogados.vagas.solides.com.br/vaga/915401</t>
-        </is>
-      </c>
-      <c r="G111" s="4" t="inlineStr">
-        <is>
-          <t>Assistente de Controladoria Juridica (PJ)</t>
-        </is>
-      </c>
-      <c r="H111" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="I111" s="4" t="inlineStr">
-        <is>
-          <t>https://to.indeed.com/aay7xrjqdxpw</t>
-        </is>
-      </c>
-      <c r="J111" s="4" t="inlineStr">
-        <is>
-          <t>"REALIZAR CANDIDATURA NO LINK: https://reisadvogados.vagas.solides.com.br/vaga/915401"</t>
-        </is>
-      </c>
-      <c r="K111" s="4" t="inlineStr">
-        <is>
-          <t>Candidatura so pelo link proprio, nao pelo Indeed.</t>
-        </is>
-      </c>
-      <c r="L111" s="4" t="inlineStr">
-        <is>
-          <t>Descricao completa da vaga no Indeed (get_job_details)</t>
-        </is>
-      </c>
-    </row>
+    <row r="111" ht="62" customHeight="1"/>
   </sheetData>
   <autoFilter ref="A1:L111"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>